<commit_message>
Restyle 5 analytical sheets with distinct colour palettes
Product Performance: rose/crimson  |  Pareto: deep indigo
Cohort Retention: amber heatmap    |  Channel ROI: emerald green
RFM Segments: cyan/sky-blue with per-tier badge colours
</commit_message>
<xml_diff>
--- a/GA4_Intelligence_Hub_v3_Final.xlsx
+++ b/GA4_Intelligence_Hub_v3_Final.xlsx
@@ -40,7 +40,7 @@
     <numFmt numFmtId="167" formatCode="0.00&quot;kg&quot;"/>
     <numFmt numFmtId="168" formatCode="0.0"/>
   </numFmts>
-  <fonts count="89">
+  <fonts count="93">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -394,7 +394,7 @@
     <font>
       <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="0078350F"/>
+      <color rgb="009D174D"/>
       <sz val="9"/>
     </font>
     <font>
@@ -411,19 +411,19 @@
     </font>
     <font>
       <name val="Calibri"/>
-      <color rgb="000E7490"/>
+      <color rgb="00BE185D"/>
       <sz val="9"/>
     </font>
     <font>
       <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="00166534"/>
+      <color rgb="0015803D"/>
       <sz val="9"/>
     </font>
     <font>
       <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="00991B1B"/>
+      <color rgb="009F1239"/>
       <sz val="9"/>
     </font>
     <font>
@@ -447,13 +447,25 @@
     <font>
       <name val="Calibri"/>
       <i val="1"/>
-      <color rgb="0014532D"/>
+      <color rgb="00312E81"/>
       <sz val="10"/>
     </font>
     <font>
       <name val="Calibri"/>
       <b val="1"/>
+      <color rgb="004F46E5"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
       <color rgb="0014532D"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="003730A3"/>
       <sz val="9"/>
     </font>
     <font>
@@ -464,7 +476,7 @@
     <font>
       <name val="Calibri"/>
       <i val="1"/>
-      <color rgb="000F4C75"/>
+      <color rgb="0078350F"/>
       <sz val="10"/>
     </font>
     <font>
@@ -480,7 +492,7 @@
     </font>
     <font>
       <name val="Calibri"/>
-      <color rgb="000F4C75"/>
+      <color rgb="0078350F"/>
       <sz val="9"/>
     </font>
     <font>
@@ -492,14 +504,8 @@
     <font>
       <name val="Calibri"/>
       <i val="1"/>
-      <color rgb="007C2D12"/>
+      <color rgb="00064E3B"/>
       <sz val="10"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <b val="1"/>
-      <color rgb="009A3412"/>
-      <sz val="9"/>
     </font>
     <font>
       <name val="Calibri"/>
@@ -513,6 +519,12 @@
     </font>
     <font>
       <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00065F46"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
       <color rgb="001D4ED8"/>
       <sz val="9"/>
     </font>
@@ -523,26 +535,38 @@
     </font>
     <font>
       <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00991B1B"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
       <i val="1"/>
-      <color rgb="004C1D95"/>
+      <color rgb="000E4F6A"/>
       <sz val="10"/>
     </font>
     <font>
       <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="004C1D95"/>
+      <color rgb="000E4F6A"/>
       <sz val="9"/>
     </font>
     <font>
       <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="00312E81"/>
+      <color rgb="000E7490"/>
       <sz val="9"/>
     </font>
     <font>
       <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="00065F46"/>
+      <color rgb="00166534"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00B45309"/>
       <sz val="9"/>
     </font>
     <font>
@@ -551,7 +575,7 @@
       <sz val="9"/>
     </font>
   </fonts>
-  <fills count="63">
+  <fills count="66">
     <fill>
       <patternFill/>
     </fill>
@@ -770,7 +794,17 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="001E3A5F"/>
+        <fgColor rgb="00881337"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FCE7F3"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF1F2"/>
       </patternFill>
     </fill>
     <fill>
@@ -780,7 +814,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="0014532D"/>
+        <fgColor rgb="001E3A5F"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00312E81"/>
       </patternFill>
     </fill>
     <fill>
@@ -790,32 +829,17 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="000F4C75"/>
+        <fgColor rgb="00EEF2FF"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00F0F9FF"/>
+        <fgColor rgb="00B45309"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="000369A1"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="000EA5E9"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="007DD3FC"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00BAE6FD"/>
+        <fgColor rgb="00FBBF24"/>
       </patternFill>
     </fill>
     <fill>
@@ -825,12 +849,27 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="007C2D12"/>
+        <fgColor rgb="00ECFDF5"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFEDD5"/>
+        <fgColor rgb="000E4F6A"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00CFFAFE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00155E75"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00ECFEFF"/>
       </patternFill>
     </fill>
     <fill>
@@ -840,7 +879,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00A78BFA"/>
+        <fgColor rgb="000E7490"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="0067E8F9"/>
       </patternFill>
     </fill>
     <fill>
@@ -855,12 +899,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00DDD6FE"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00C4B5FD"/>
+        <fgColor rgb="0022D3EE"/>
       </patternFill>
     </fill>
   </fills>
@@ -914,7 +953,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="382">
+  <cellXfs count="388">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -1706,7 +1745,7 @@
     <xf numFmtId="0" fontId="3" fillId="44" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="61" fillId="10" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="61" fillId="45" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="62" fillId="17" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -1733,43 +1772,43 @@
     <xf numFmtId="166" fontId="64" fillId="17" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="62" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="62" fillId="46" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="63" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="63" fillId="46" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="64" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="64" fillId="46" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="41" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="41" fillId="46" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="65" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="65" fillId="46" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="3" fontId="41" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="3" fontId="41" fillId="46" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="41" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="41" fillId="46" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="64" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="166" fontId="64" fillId="46" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="65" fillId="17" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="66" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="66" fillId="46" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="67" fillId="45" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="67" fillId="47" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="41" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="41" fillId="46" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="65" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="65" fillId="46" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="41" fillId="17" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -1781,271 +1820,289 @@
     <xf numFmtId="0" fontId="68" fillId="17" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="68" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="68" fillId="46" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="44" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="44" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="48" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="48" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="69" fillId="44" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="69" fillId="48" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="3" fontId="69" fillId="44" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="3" fontId="69" fillId="48" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="46" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="14" fillId="49" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="70" fillId="47" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="70" fillId="50" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="46" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="49" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="71" fillId="17" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="72" fillId="17" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="73" fillId="17" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="166" fontId="41" fillId="17" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="62" fillId="17" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="166" fontId="71" fillId="17" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="9" fontId="42" fillId="17" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="72" fillId="17" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="74" fillId="17" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="62" fillId="20" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="73" fillId="17" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="71" fillId="20" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="71" fillId="51" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="72" fillId="51" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="65" fillId="20" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="73" fillId="51" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="41" fillId="20" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="166" fontId="41" fillId="51" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="62" fillId="20" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="166" fontId="71" fillId="51" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="9" fontId="42" fillId="20" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="9" fontId="42" fillId="51" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="72" fillId="20" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="74" fillId="51" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="65" fillId="20" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="73" fillId="51" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="41" fillId="20" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="41" fillId="51" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="68" fillId="20" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="68" fillId="51" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="48" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="14" fillId="43" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="73" fillId="25" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="75" fillId="10" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="48" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="43" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="74" fillId="18" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="76" fillId="37" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="3" fontId="41" fillId="49" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="3" fontId="41" fillId="38" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="9" fontId="3" fillId="50" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="9" fontId="3" fillId="52" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="9" fontId="75" fillId="50" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="9" fontId="77" fillId="52" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="9" fontId="75" fillId="51" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="9" fontId="77" fillId="9" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="9" fontId="76" fillId="52" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="9" fontId="78" fillId="53" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="9" fontId="76" fillId="53" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="9" fontId="78" fillId="37" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="54" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="77" fillId="12" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="79" fillId="12" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="55" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="14" fillId="29" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="78" fillId="56" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="80" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="55" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="29" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="79" fillId="17" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="19" fillId="17" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="81" fillId="17" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="82" fillId="17" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="10" fontId="82" fillId="17" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="83" fillId="17" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="84" fillId="17" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="41" fillId="17" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="79" fillId="17" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="166" fontId="19" fillId="17" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="79" fillId="21" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="19" fillId="55" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="81" fillId="21" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="82" fillId="55" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="65" fillId="21" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="83" fillId="55" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="3" fontId="41" fillId="21" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="3" fontId="41" fillId="55" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="10" fontId="82" fillId="21" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="10" fontId="84" fillId="55" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="41" fillId="21" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="49" fontId="41" fillId="55" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="41" fillId="21" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="41" fillId="55" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="79" fillId="21" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="166" fontId="19" fillId="55" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="83" fillId="17" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="85" fillId="17" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="83" fillId="21" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="86" fillId="17" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="85" fillId="55" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="65" fillId="21" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="83" fillId="55" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="41" fillId="21" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="41" fillId="55" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="66" fillId="21" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="86" fillId="55" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="55" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="29" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="55" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="69" fillId="55" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="29" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="69" fillId="29" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="3" fontId="69" fillId="55" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="3" fontId="69" fillId="29" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="31" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="14" fillId="56" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="84" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="87" fillId="57" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="31" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="56" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="85" fillId="17" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="88" fillId="17" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="86" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="89" fillId="57" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="31" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="58" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="30" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="65" fillId="17" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="90" fillId="17" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="16" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="85" fillId="34" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="56" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="88" fillId="59" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="3" fontId="41" fillId="34" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="3" fontId="41" fillId="59" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="65" fillId="34" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="90" fillId="59" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="41" fillId="34" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="41" fillId="59" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="60" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="61" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="83" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="68" fillId="62" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="68" fillId="63" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="68" fillId="64" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="65" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="62" fillId="18" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="68" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="68" fillId="57" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="91" fillId="10" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="68" fillId="18" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="57" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="86" fillId="23" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="87" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="68" fillId="58" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="68" fillId="59" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="68" fillId="60" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="58" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="62" fillId="18" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="68" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="68" fillId="61" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="10" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="68" fillId="18" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="62" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="66" fillId="23" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="31" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="56" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="41" fillId="12" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="88" fillId="12" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="92" fillId="12" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="41" fillId="12" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -15109,327 +15166,327 @@
       </c>
     </row>
     <row r="5" ht="17" customHeight="1">
-      <c r="A5" s="266" t="n">
+      <c r="A5" s="298" t="n">
         <v>1</v>
       </c>
-      <c r="B5" s="298" t="inlineStr">
+      <c r="B5" s="299" t="inlineStr">
         <is>
           <t>Google Unisex Eco Tee</t>
         </is>
       </c>
-      <c r="C5" s="270" t="n">
+      <c r="C5" s="300" t="n">
         <v>150200</v>
       </c>
-      <c r="D5" s="299" t="n">
+      <c r="D5" s="301" t="n">
         <v>0.1684838695203482</v>
       </c>
-      <c r="E5" s="300" t="n">
+      <c r="E5" s="302" t="n">
         <v>0.1684838695203482</v>
       </c>
-      <c r="F5" s="301" t="n">
+      <c r="F5" s="303" t="n">
         <v>0.8</v>
       </c>
-      <c r="G5" s="302" t="inlineStr">
+      <c r="G5" s="304" t="inlineStr">
         <is>
           <t>Apparel</t>
         </is>
       </c>
-      <c r="H5" s="282" t="inlineStr">
+      <c r="H5" s="305" t="inlineStr">
         <is>
           <t>Core (80%)</t>
         </is>
       </c>
     </row>
     <row r="6" ht="17" customHeight="1">
-      <c r="A6" s="303" t="n">
+      <c r="A6" s="306" t="n">
         <v>2</v>
       </c>
-      <c r="B6" s="304" t="inlineStr">
+      <c r="B6" s="307" t="inlineStr">
         <is>
           <t>YouTube Brand Hoodie</t>
         </is>
       </c>
-      <c r="C6" s="305" t="n">
+      <c r="C6" s="308" t="n">
         <v>103980</v>
       </c>
-      <c r="D6" s="306" t="n">
+      <c r="D6" s="309" t="n">
         <v>0.1166375016825952</v>
       </c>
-      <c r="E6" s="307" t="n">
+      <c r="E6" s="310" t="n">
         <v>0.2851213712029435</v>
       </c>
-      <c r="F6" s="308" t="n">
+      <c r="F6" s="311" t="n">
         <v>0.8</v>
       </c>
-      <c r="G6" s="309" t="inlineStr">
+      <c r="G6" s="312" t="inlineStr">
         <is>
           <t>Apparel</t>
         </is>
       </c>
-      <c r="H6" s="310" t="inlineStr">
+      <c r="H6" s="313" t="inlineStr">
         <is>
           <t>Core (80%)</t>
         </is>
       </c>
     </row>
     <row r="7" ht="17" customHeight="1">
-      <c r="A7" s="266" t="n">
+      <c r="A7" s="298" t="n">
         <v>3</v>
       </c>
-      <c r="B7" s="298" t="inlineStr">
+      <c r="B7" s="299" t="inlineStr">
         <is>
           <t>Google Zip-Up Hoodie</t>
         </is>
       </c>
-      <c r="C7" s="270" t="n">
+      <c r="C7" s="300" t="n">
         <v>88986</v>
       </c>
-      <c r="D7" s="299" t="n">
+      <c r="D7" s="301" t="n">
         <v>0.09981827971463185</v>
       </c>
-      <c r="E7" s="300" t="n">
+      <c r="E7" s="302" t="n">
         <v>0.3849396509175753</v>
       </c>
-      <c r="F7" s="301" t="n">
+      <c r="F7" s="303" t="n">
         <v>0.8</v>
       </c>
-      <c r="G7" s="302" t="inlineStr">
+      <c r="G7" s="304" t="inlineStr">
         <is>
           <t>Apparel</t>
         </is>
       </c>
-      <c r="H7" s="282" t="inlineStr">
+      <c r="H7" s="305" t="inlineStr">
         <is>
           <t>Core (80%)</t>
         </is>
       </c>
     </row>
     <row r="8" ht="17" customHeight="1">
-      <c r="A8" s="303" t="n">
+      <c r="A8" s="306" t="n">
         <v>4</v>
       </c>
-      <c r="B8" s="304" t="inlineStr">
+      <c r="B8" s="307" t="inlineStr">
         <is>
           <t>Google Fleece Jacket</t>
         </is>
       </c>
-      <c r="C8" s="305" t="n">
+      <c r="C8" s="308" t="n">
         <v>79990</v>
       </c>
-      <c r="D8" s="306" t="n">
+      <c r="D8" s="309" t="n">
         <v>0.08972719522591645</v>
       </c>
-      <c r="E8" s="307" t="n">
+      <c r="E8" s="310" t="n">
         <v>0.4746668461434917</v>
       </c>
-      <c r="F8" s="308" t="n">
+      <c r="F8" s="311" t="n">
         <v>0.8</v>
       </c>
-      <c r="G8" s="309" t="inlineStr">
+      <c r="G8" s="312" t="inlineStr">
         <is>
           <t>Apparel</t>
         </is>
       </c>
-      <c r="H8" s="310" t="inlineStr">
+      <c r="H8" s="313" t="inlineStr">
         <is>
           <t>Core (80%)</t>
         </is>
       </c>
     </row>
     <row r="9" ht="17" customHeight="1">
-      <c r="A9" s="266" t="n">
+      <c r="A9" s="298" t="n">
         <v>5</v>
       </c>
-      <c r="B9" s="298" t="inlineStr">
+      <c r="B9" s="299" t="inlineStr">
         <is>
           <t>Google Polo Shirt White</t>
         </is>
       </c>
-      <c r="C9" s="270" t="n">
+      <c r="C9" s="300" t="n">
         <v>67982</v>
       </c>
-      <c r="D9" s="299" t="n">
+      <c r="D9" s="301" t="n">
         <v>0.07625745950554134</v>
       </c>
-      <c r="E9" s="300" t="n">
+      <c r="E9" s="302" t="n">
         <v>0.5509243056490331</v>
       </c>
-      <c r="F9" s="301" t="n">
+      <c r="F9" s="303" t="n">
         <v>0.8</v>
       </c>
-      <c r="G9" s="302" t="inlineStr">
+      <c r="G9" s="304" t="inlineStr">
         <is>
           <t>Apparel</t>
         </is>
       </c>
-      <c r="H9" s="282" t="inlineStr">
+      <c r="H9" s="305" t="inlineStr">
         <is>
           <t>Core (80%)</t>
         </is>
       </c>
     </row>
     <row r="10" ht="17" customHeight="1">
-      <c r="A10" s="303" t="n">
+      <c r="A10" s="306" t="n">
         <v>6</v>
       </c>
-      <c r="B10" s="304" t="inlineStr">
+      <c r="B10" s="307" t="inlineStr">
         <is>
           <t>Google Sport Duffel</t>
         </is>
       </c>
-      <c r="C10" s="305" t="n">
+      <c r="C10" s="308" t="n">
         <v>55487</v>
       </c>
-      <c r="D10" s="306" t="n">
+      <c r="D10" s="309" t="n">
         <v>0.06224144119890519</v>
       </c>
-      <c r="E10" s="307" t="n">
+      <c r="E10" s="310" t="n">
         <v>0.6131657468479382</v>
       </c>
-      <c r="F10" s="308" t="n">
+      <c r="F10" s="311" t="n">
         <v>0.8</v>
       </c>
-      <c r="G10" s="309" t="inlineStr">
+      <c r="G10" s="312" t="inlineStr">
         <is>
           <t>Bags</t>
         </is>
       </c>
-      <c r="H10" s="310" t="inlineStr">
+      <c r="H10" s="313" t="inlineStr">
         <is>
           <t>Core (80%)</t>
         </is>
       </c>
     </row>
     <row r="11" ht="17" customHeight="1">
-      <c r="A11" s="266" t="n">
+      <c r="A11" s="298" t="n">
         <v>7</v>
       </c>
-      <c r="B11" s="298" t="inlineStr">
+      <c r="B11" s="299" t="inlineStr">
         <is>
           <t>Google Stainless Steel Bottle</t>
         </is>
       </c>
-      <c r="C11" s="270" t="n">
+      <c r="C11" s="300" t="n">
         <v>45818</v>
       </c>
-      <c r="D11" s="299" t="n">
+      <c r="D11" s="301" t="n">
         <v>0.05139543231480235</v>
       </c>
-      <c r="E11" s="300" t="n">
+      <c r="E11" s="302" t="n">
         <v>0.6645611791627406</v>
       </c>
-      <c r="F11" s="301" t="n">
+      <c r="F11" s="303" t="n">
         <v>0.8</v>
       </c>
-      <c r="G11" s="302" t="inlineStr">
+      <c r="G11" s="304" t="inlineStr">
         <is>
           <t>Drinkware</t>
         </is>
       </c>
-      <c r="H11" s="282" t="inlineStr">
+      <c r="H11" s="305" t="inlineStr">
         <is>
           <t>Core (80%)</t>
         </is>
       </c>
     </row>
     <row r="12" ht="17" customHeight="1">
-      <c r="A12" s="303" t="n">
+      <c r="A12" s="306" t="n">
         <v>8</v>
       </c>
-      <c r="B12" s="304" t="inlineStr">
+      <c r="B12" s="307" t="inlineStr">
         <is>
           <t>Google Leather Journal</t>
         </is>
       </c>
-      <c r="C12" s="305" t="n">
+      <c r="C12" s="308" t="n">
         <v>38987</v>
       </c>
-      <c r="D12" s="306" t="n">
+      <c r="D12" s="309" t="n">
         <v>0.04373289361511195</v>
       </c>
-      <c r="E12" s="307" t="n">
+      <c r="E12" s="310" t="n">
         <v>0.7082940727778525</v>
       </c>
-      <c r="F12" s="308" t="n">
+      <c r="F12" s="311" t="n">
         <v>0.8</v>
       </c>
-      <c r="G12" s="309" t="inlineStr">
+      <c r="G12" s="312" t="inlineStr">
         <is>
           <t>Office</t>
         </is>
       </c>
-      <c r="H12" s="310" t="inlineStr">
+      <c r="H12" s="313" t="inlineStr">
         <is>
           <t>Core (80%)</t>
         </is>
       </c>
     </row>
     <row r="13" ht="17" customHeight="1">
-      <c r="A13" s="266" t="n">
+      <c r="A13" s="298" t="n">
         <v>9</v>
       </c>
-      <c r="B13" s="298" t="inlineStr">
+      <c r="B13" s="299" t="inlineStr">
         <is>
           <t>Pixel Buds Tote Bag</t>
         </is>
       </c>
-      <c r="C13" s="270" t="n">
+      <c r="C13" s="300" t="n">
         <v>33985</v>
       </c>
-      <c r="D13" s="299" t="n">
+      <c r="D13" s="301" t="n">
         <v>0.03812199937183111</v>
       </c>
-      <c r="E13" s="300" t="n">
+      <c r="E13" s="302" t="n">
         <v>0.7464160721496836</v>
       </c>
-      <c r="F13" s="301" t="n">
+      <c r="F13" s="303" t="n">
         <v>0.8</v>
       </c>
-      <c r="G13" s="302" t="inlineStr">
+      <c r="G13" s="304" t="inlineStr">
         <is>
           <t>Bags</t>
         </is>
       </c>
-      <c r="H13" s="282" t="inlineStr">
+      <c r="H13" s="305" t="inlineStr">
         <is>
           <t>Core (80%)</t>
         </is>
       </c>
     </row>
     <row r="14" ht="17" customHeight="1">
-      <c r="A14" s="303" t="n">
+      <c r="A14" s="306" t="n">
         <v>10</v>
       </c>
-      <c r="B14" s="304" t="inlineStr">
+      <c r="B14" s="307" t="inlineStr">
         <is>
           <t>Google Embroidered Cap</t>
         </is>
       </c>
-      <c r="C14" s="305" t="n">
+      <c r="C14" s="308" t="n">
         <v>29386</v>
       </c>
-      <c r="D14" s="306" t="n">
+      <c r="D14" s="309" t="n">
         <v>0.03296316238165747</v>
       </c>
-      <c r="E14" s="307" t="n">
+      <c r="E14" s="310" t="n">
         <v>0.7793792345313411</v>
       </c>
-      <c r="F14" s="308" t="n">
+      <c r="F14" s="311" t="n">
         <v>0.8</v>
       </c>
-      <c r="G14" s="309" t="inlineStr">
+      <c r="G14" s="312" t="inlineStr">
         <is>
           <t>Apparel</t>
         </is>
       </c>
-      <c r="H14" s="310" t="inlineStr">
+      <c r="H14" s="313" t="inlineStr">
         <is>
           <t>Core (80%)</t>
         </is>
       </c>
     </row>
     <row r="15" ht="17" customHeight="1">
-      <c r="A15" s="266" t="n">
+      <c r="A15" s="298" t="n">
         <v>11</v>
       </c>
       <c r="B15" s="287" t="inlineStr">
@@ -15437,19 +15494,19 @@
           <t>Workspace Blue Tumbler</t>
         </is>
       </c>
-      <c r="C15" s="270" t="n">
+      <c r="C15" s="300" t="n">
         <v>25186</v>
       </c>
-      <c r="D15" s="299" t="n">
+      <c r="D15" s="301" t="n">
         <v>0.02825189572396464</v>
       </c>
-      <c r="E15" s="300" t="n">
+      <c r="E15" s="302" t="n">
         <v>0.8076311302553058</v>
       </c>
-      <c r="F15" s="301" t="n">
+      <c r="F15" s="303" t="n">
         <v>0.8</v>
       </c>
-      <c r="G15" s="302" t="inlineStr">
+      <c r="G15" s="304" t="inlineStr">
         <is>
           <t>Drinkware</t>
         </is>
@@ -15461,39 +15518,39 @@
       </c>
     </row>
     <row r="16" ht="17" customHeight="1">
-      <c r="A16" s="303" t="n">
+      <c r="A16" s="306" t="n">
         <v>12</v>
       </c>
-      <c r="B16" s="311" t="inlineStr">
+      <c r="B16" s="314" t="inlineStr">
         <is>
           <t>Google Maps Tote Bag</t>
         </is>
       </c>
-      <c r="C16" s="305" t="n">
+      <c r="C16" s="308" t="n">
         <v>23987</v>
       </c>
-      <c r="D16" s="306" t="n">
+      <c r="D16" s="309" t="n">
         <v>0.026906941266209</v>
       </c>
-      <c r="E16" s="307" t="n">
+      <c r="E16" s="310" t="n">
         <v>0.8345380715215147</v>
       </c>
-      <c r="F16" s="308" t="n">
+      <c r="F16" s="311" t="n">
         <v>0.8</v>
       </c>
-      <c r="G16" s="309" t="inlineStr">
+      <c r="G16" s="312" t="inlineStr">
         <is>
           <t>Bags</t>
         </is>
       </c>
-      <c r="H16" s="312" t="inlineStr">
+      <c r="H16" s="315" t="inlineStr">
         <is>
           <t>Long Tail</t>
         </is>
       </c>
     </row>
     <row r="17" ht="17" customHeight="1">
-      <c r="A17" s="266" t="n">
+      <c r="A17" s="298" t="n">
         <v>13</v>
       </c>
       <c r="B17" s="287" t="inlineStr">
@@ -15501,19 +15558,19 @@
           <t>YouTube Music Beanie</t>
         </is>
       </c>
-      <c r="C17" s="270" t="n">
+      <c r="C17" s="300" t="n">
         <v>21587</v>
       </c>
-      <c r="D17" s="299" t="n">
+      <c r="D17" s="301" t="n">
         <v>0.02421478889038453</v>
       </c>
-      <c r="E17" s="300" t="n">
+      <c r="E17" s="302" t="n">
         <v>0.8587528604118992</v>
       </c>
-      <c r="F17" s="301" t="n">
+      <c r="F17" s="303" t="n">
         <v>0.8</v>
       </c>
-      <c r="G17" s="302" t="inlineStr">
+      <c r="G17" s="304" t="inlineStr">
         <is>
           <t>Apparel</t>
         </is>
@@ -15525,39 +15582,39 @@
       </c>
     </row>
     <row r="18" ht="17" customHeight="1">
-      <c r="A18" s="303" t="n">
+      <c r="A18" s="306" t="n">
         <v>14</v>
       </c>
-      <c r="B18" s="311" t="inlineStr">
+      <c r="B18" s="314" t="inlineStr">
         <is>
           <t>Cloud Platform Mug</t>
         </is>
       </c>
-      <c r="C18" s="305" t="n">
+      <c r="C18" s="308" t="n">
         <v>19987</v>
       </c>
-      <c r="D18" s="306" t="n">
+      <c r="D18" s="309" t="n">
         <v>0.02242002063983488</v>
       </c>
-      <c r="E18" s="307" t="n">
+      <c r="E18" s="310" t="n">
         <v>0.8811728810517341</v>
       </c>
-      <c r="F18" s="308" t="n">
+      <c r="F18" s="311" t="n">
         <v>0.8</v>
       </c>
-      <c r="G18" s="309" t="inlineStr">
+      <c r="G18" s="312" t="inlineStr">
         <is>
           <t>Drinkware</t>
         </is>
       </c>
-      <c r="H18" s="312" t="inlineStr">
+      <c r="H18" s="315" t="inlineStr">
         <is>
           <t>Long Tail</t>
         </is>
       </c>
     </row>
     <row r="19" ht="17" customHeight="1">
-      <c r="A19" s="266" t="n">
+      <c r="A19" s="298" t="n">
         <v>15</v>
       </c>
       <c r="B19" s="287" t="inlineStr">
@@ -15565,19 +15622,19 @@
           <t>Google Pixel Watch Band</t>
         </is>
       </c>
-      <c r="C19" s="270" t="n">
+      <c r="C19" s="300" t="n">
         <v>17074</v>
       </c>
-      <c r="D19" s="299" t="n">
+      <c r="D19" s="301" t="n">
         <v>0.01915242069367793</v>
       </c>
-      <c r="E19" s="300" t="n">
+      <c r="E19" s="302" t="n">
         <v>0.900325301745412</v>
       </c>
-      <c r="F19" s="301" t="n">
+      <c r="F19" s="303" t="n">
         <v>0.8</v>
       </c>
-      <c r="G19" s="302" t="inlineStr">
+      <c r="G19" s="304" t="inlineStr">
         <is>
           <t>Accessories</t>
         </is>
@@ -15589,39 +15646,39 @@
       </c>
     </row>
     <row r="20" ht="17" customHeight="1">
-      <c r="A20" s="303" t="n">
+      <c r="A20" s="306" t="n">
         <v>16</v>
       </c>
-      <c r="B20" s="311" t="inlineStr">
+      <c r="B20" s="314" t="inlineStr">
         <is>
           <t>Google Waze Plush Toy</t>
         </is>
       </c>
-      <c r="C20" s="305" t="n">
+      <c r="C20" s="308" t="n">
         <v>15391</v>
       </c>
-      <c r="D20" s="306" t="n">
+      <c r="D20" s="309" t="n">
         <v>0.01726454884013102</v>
       </c>
-      <c r="E20" s="307" t="n">
+      <c r="E20" s="310" t="n">
         <v>0.9175898505855431</v>
       </c>
-      <c r="F20" s="308" t="n">
+      <c r="F20" s="311" t="n">
         <v>0.8</v>
       </c>
-      <c r="G20" s="309" t="inlineStr">
+      <c r="G20" s="312" t="inlineStr">
         <is>
           <t>Accessories</t>
         </is>
       </c>
-      <c r="H20" s="312" t="inlineStr">
+      <c r="H20" s="315" t="inlineStr">
         <is>
           <t>Long Tail</t>
         </is>
       </c>
     </row>
     <row r="21" ht="17" customHeight="1">
-      <c r="A21" s="266" t="n">
+      <c r="A21" s="298" t="n">
         <v>17</v>
       </c>
       <c r="B21" s="287" t="inlineStr">
@@ -15629,19 +15686,19 @@
           <t>Android Plush Toy</t>
         </is>
       </c>
-      <c r="C21" s="270" t="n">
+      <c r="C21" s="300" t="n">
         <v>13491</v>
       </c>
-      <c r="D21" s="299" t="n">
+      <c r="D21" s="301" t="n">
         <v>0.01513326154260331</v>
       </c>
-      <c r="E21" s="300" t="n">
+      <c r="E21" s="302" t="n">
         <v>0.9327231121281464</v>
       </c>
-      <c r="F21" s="301" t="n">
+      <c r="F21" s="303" t="n">
         <v>0.8</v>
       </c>
-      <c r="G21" s="302" t="inlineStr">
+      <c r="G21" s="304" t="inlineStr">
         <is>
           <t>Accessories</t>
         </is>
@@ -15653,39 +15710,39 @@
       </c>
     </row>
     <row r="22" ht="17" customHeight="1">
-      <c r="A22" s="303" t="n">
+      <c r="A22" s="306" t="n">
         <v>18</v>
       </c>
-      <c r="B22" s="311" t="inlineStr">
+      <c r="B22" s="314" t="inlineStr">
         <is>
           <t>Google Spiral Notebook</t>
         </is>
       </c>
-      <c r="C22" s="305" t="n">
+      <c r="C22" s="308" t="n">
         <v>11691</v>
       </c>
-      <c r="D22" s="306" t="n">
+      <c r="D22" s="309" t="n">
         <v>0.01311414726073496</v>
       </c>
-      <c r="E22" s="307" t="n">
+      <c r="E22" s="310" t="n">
         <v>0.9458372593888814</v>
       </c>
-      <c r="F22" s="308" t="n">
+      <c r="F22" s="311" t="n">
         <v>0.8</v>
       </c>
-      <c r="G22" s="309" t="inlineStr">
+      <c r="G22" s="312" t="inlineStr">
         <is>
           <t>Office</t>
         </is>
       </c>
-      <c r="H22" s="312" t="inlineStr">
+      <c r="H22" s="315" t="inlineStr">
         <is>
           <t>Long Tail</t>
         </is>
       </c>
     </row>
     <row r="23" ht="17" customHeight="1">
-      <c r="A23" s="266" t="n">
+      <c r="A23" s="298" t="n">
         <v>19</v>
       </c>
       <c r="B23" s="287" t="inlineStr">
@@ -15693,19 +15750,19 @@
           <t>Google Classic Tee Navy</t>
         </is>
       </c>
-      <c r="C23" s="270" t="n">
+      <c r="C23" s="300" t="n">
         <v>10106</v>
       </c>
-      <c r="D23" s="299" t="n">
+      <c r="D23" s="301" t="n">
         <v>0.01133620496253421</v>
       </c>
-      <c r="E23" s="300" t="n">
+      <c r="E23" s="302" t="n">
         <v>0.9571734643514156</v>
       </c>
-      <c r="F23" s="301" t="n">
+      <c r="F23" s="303" t="n">
         <v>0.8</v>
       </c>
-      <c r="G23" s="302" t="inlineStr">
+      <c r="G23" s="304" t="inlineStr">
         <is>
           <t>Apparel</t>
         </is>
@@ -15717,39 +15774,39 @@
       </c>
     </row>
     <row r="24" ht="17" customHeight="1">
-      <c r="A24" s="303" t="n">
+      <c r="A24" s="306" t="n">
         <v>20</v>
       </c>
-      <c r="B24" s="311" t="inlineStr">
+      <c r="B24" s="314" t="inlineStr">
         <is>
           <t>Google Sunglasses</t>
         </is>
       </c>
-      <c r="C24" s="305" t="n">
+      <c r="C24" s="308" t="n">
         <v>8908</v>
       </c>
-      <c r="D24" s="306" t="n">
+      <c r="D24" s="309" t="n">
         <v>0.009992372234935164</v>
       </c>
-      <c r="E24" s="307" t="n">
+      <c r="E24" s="310" t="n">
         <v>0.9671658365863508</v>
       </c>
-      <c r="F24" s="308" t="n">
+      <c r="F24" s="311" t="n">
         <v>0.8</v>
       </c>
-      <c r="G24" s="309" t="inlineStr">
+      <c r="G24" s="312" t="inlineStr">
         <is>
           <t>Accessories</t>
         </is>
       </c>
-      <c r="H24" s="312" t="inlineStr">
+      <c r="H24" s="315" t="inlineStr">
         <is>
           <t>Long Tail</t>
         </is>
       </c>
     </row>
     <row r="25" ht="17" customHeight="1">
-      <c r="A25" s="266" t="n">
+      <c r="A25" s="298" t="n">
         <v>21</v>
       </c>
       <c r="B25" s="287" t="inlineStr">
@@ -15757,19 +15814,19 @@
           <t>Chrome Dino Enamel Pin</t>
         </is>
       </c>
-      <c r="C25" s="270" t="n">
+      <c r="C25" s="300" t="n">
         <v>7993</v>
       </c>
-      <c r="D25" s="299" t="n">
+      <c r="D25" s="301" t="n">
         <v>0.008965989141652085</v>
       </c>
-      <c r="E25" s="300" t="n">
+      <c r="E25" s="302" t="n">
         <v>0.9761318257280028</v>
       </c>
-      <c r="F25" s="301" t="n">
+      <c r="F25" s="303" t="n">
         <v>0.8</v>
       </c>
-      <c r="G25" s="302" t="inlineStr">
+      <c r="G25" s="304" t="inlineStr">
         <is>
           <t>Accessories</t>
         </is>
@@ -15781,39 +15838,39 @@
       </c>
     </row>
     <row r="26" ht="17" customHeight="1">
-      <c r="A26" s="303" t="n">
+      <c r="A26" s="306" t="n">
         <v>22</v>
       </c>
-      <c r="B26" s="311" t="inlineStr">
+      <c r="B26" s="314" t="inlineStr">
         <is>
           <t>Android Snapback Hat</t>
         </is>
       </c>
-      <c r="C26" s="305" t="n">
+      <c r="C26" s="308" t="n">
         <v>6596</v>
       </c>
-      <c r="D26" s="306" t="n">
+      <c r="D26" s="309" t="n">
         <v>0.007398932112890923</v>
       </c>
-      <c r="E26" s="307" t="n">
+      <c r="E26" s="310" t="n">
         <v>0.9835307578408937</v>
       </c>
-      <c r="F26" s="308" t="n">
+      <c r="F26" s="311" t="n">
         <v>0.8</v>
       </c>
-      <c r="G26" s="309" t="inlineStr">
+      <c r="G26" s="312" t="inlineStr">
         <is>
           <t>Apparel</t>
         </is>
       </c>
-      <c r="H26" s="312" t="inlineStr">
+      <c r="H26" s="315" t="inlineStr">
         <is>
           <t>Long Tail</t>
         </is>
       </c>
     </row>
     <row r="27" ht="17" customHeight="1">
-      <c r="A27" s="266" t="n">
+      <c r="A27" s="298" t="n">
         <v>23</v>
       </c>
       <c r="B27" s="287" t="inlineStr">
@@ -15821,19 +15878,19 @@
           <t>Google Phone Stand</t>
         </is>
       </c>
-      <c r="C27" s="270" t="n">
+      <c r="C27" s="300" t="n">
         <v>5997</v>
       </c>
-      <c r="D27" s="299" t="n">
+      <c r="D27" s="301" t="n">
         <v>0.006727015749091399</v>
       </c>
-      <c r="E27" s="300" t="n">
+      <c r="E27" s="302" t="n">
         <v>0.9902577735899851</v>
       </c>
-      <c r="F27" s="301" t="n">
+      <c r="F27" s="303" t="n">
         <v>0.8</v>
       </c>
-      <c r="G27" s="302" t="inlineStr">
+      <c r="G27" s="304" t="inlineStr">
         <is>
           <t>Office</t>
         </is>
@@ -15845,39 +15902,39 @@
       </c>
     </row>
     <row r="28" ht="17" customHeight="1">
-      <c r="A28" s="303" t="n">
+      <c r="A28" s="306" t="n">
         <v>24</v>
       </c>
-      <c r="B28" s="311" t="inlineStr">
+      <c r="B28" s="314" t="inlineStr">
         <is>
           <t>BigQuery Sticker Pack</t>
         </is>
       </c>
-      <c r="C28" s="305" t="n">
+      <c r="C28" s="308" t="n">
         <v>4691</v>
       </c>
-      <c r="D28" s="306" t="n">
+      <c r="D28" s="309" t="n">
         <v>0.005262036164580248</v>
       </c>
-      <c r="E28" s="307" t="n">
+      <c r="E28" s="310" t="n">
         <v>0.9955198097545653</v>
       </c>
-      <c r="F28" s="308" t="n">
+      <c r="F28" s="311" t="n">
         <v>0.8</v>
       </c>
-      <c r="G28" s="309" t="inlineStr">
+      <c r="G28" s="312" t="inlineStr">
         <is>
           <t>Office</t>
         </is>
       </c>
-      <c r="H28" s="312" t="inlineStr">
+      <c r="H28" s="315" t="inlineStr">
         <is>
           <t>Long Tail</t>
         </is>
       </c>
     </row>
     <row r="29" ht="17" customHeight="1">
-      <c r="A29" s="266" t="n">
+      <c r="A29" s="298" t="n">
         <v>25</v>
       </c>
       <c r="B29" s="287" t="inlineStr">
@@ -15885,19 +15942,19 @@
           <t>Chrome Enterprise Lanyard</t>
         </is>
       </c>
-      <c r="C29" s="270" t="n">
+      <c r="C29" s="300" t="n">
         <v>3994</v>
       </c>
-      <c r="D29" s="299" t="n">
+      <c r="D29" s="301" t="n">
         <v>0.004480190245434558</v>
       </c>
-      <c r="E29" s="300" t="n">
+      <c r="E29" s="302" t="n">
         <v>0.9999999999999999</v>
       </c>
-      <c r="F29" s="301" t="n">
+      <c r="F29" s="303" t="n">
         <v>0.8</v>
       </c>
-      <c r="G29" s="302" t="inlineStr">
+      <c r="G29" s="304" t="inlineStr">
         <is>
           <t>Accessories</t>
         </is>
@@ -15944,14 +16001,14 @@
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
-      <c r="A1" s="313" t="inlineStr">
+      <c r="A1" s="316" t="inlineStr">
         <is>
           <t>COHORT RETENTION ANALYSIS  ·  Monthly Cohorts  ·  GA4 Intelligence Hub</t>
         </is>
       </c>
     </row>
     <row r="2" ht="16" customHeight="1">
-      <c r="A2" s="314" t="inlineStr">
+      <c r="A2" s="317" t="inlineStr">
         <is>
           <t>Insight: Month-0 retention = 100%  ·  Month-1 avg = 42%  ·  Month-3 avg = 28%  ·  Month-6 avg = 19%  ·  Month-12 avg = 11%</t>
         </is>
@@ -15959,543 +16016,543 @@
     </row>
     <row r="3" ht="6" customHeight="1"/>
     <row r="4" ht="20" customHeight="1">
-      <c r="A4" s="315" t="inlineStr">
+      <c r="A4" s="318" t="inlineStr">
         <is>
           <t>Cohort</t>
         </is>
       </c>
-      <c r="B4" s="315" t="inlineStr">
+      <c r="B4" s="318" t="inlineStr">
         <is>
           <t>New Users</t>
         </is>
       </c>
-      <c r="C4" s="315" t="inlineStr">
+      <c r="C4" s="318" t="inlineStr">
         <is>
           <t>M+0</t>
         </is>
       </c>
-      <c r="D4" s="315" t="inlineStr">
+      <c r="D4" s="318" t="inlineStr">
         <is>
           <t>M+1</t>
         </is>
       </c>
-      <c r="E4" s="315" t="inlineStr">
+      <c r="E4" s="318" t="inlineStr">
         <is>
           <t>M+2</t>
         </is>
       </c>
-      <c r="F4" s="315" t="inlineStr">
+      <c r="F4" s="318" t="inlineStr">
         <is>
           <t>M+3</t>
         </is>
       </c>
-      <c r="G4" s="315" t="inlineStr">
+      <c r="G4" s="318" t="inlineStr">
         <is>
           <t>M+4</t>
         </is>
       </c>
-      <c r="H4" s="315" t="inlineStr">
+      <c r="H4" s="318" t="inlineStr">
         <is>
           <t>M+5</t>
         </is>
       </c>
-      <c r="I4" s="315" t="inlineStr">
+      <c r="I4" s="318" t="inlineStr">
         <is>
           <t>M+6</t>
         </is>
       </c>
-      <c r="J4" s="315" t="inlineStr">
+      <c r="J4" s="318" t="inlineStr">
         <is>
           <t>M+7</t>
         </is>
       </c>
-      <c r="K4" s="315" t="inlineStr">
+      <c r="K4" s="318" t="inlineStr">
         <is>
           <t>M+8</t>
         </is>
       </c>
-      <c r="L4" s="315" t="inlineStr">
+      <c r="L4" s="318" t="inlineStr">
         <is>
           <t>M+9</t>
         </is>
       </c>
-      <c r="M4" s="315" t="inlineStr">
+      <c r="M4" s="318" t="inlineStr">
         <is>
           <t>M+10</t>
         </is>
       </c>
-      <c r="N4" s="315" t="inlineStr">
+      <c r="N4" s="318" t="inlineStr">
         <is>
           <t>M+11</t>
         </is>
       </c>
-      <c r="O4" s="315" t="inlineStr">
+      <c r="O4" s="318" t="inlineStr">
         <is>
           <t>M+12</t>
         </is>
       </c>
     </row>
     <row r="5" ht="18" customHeight="1">
-      <c r="A5" s="316" t="inlineStr">
+      <c r="A5" s="319" t="inlineStr">
         <is>
           <t>Nov-20</t>
         </is>
       </c>
-      <c r="B5" s="317" t="n">
+      <c r="B5" s="320" t="n">
         <v>3800</v>
       </c>
-      <c r="C5" s="318" t="n">
+      <c r="C5" s="321" t="n">
         <v>1</v>
       </c>
-      <c r="D5" s="319" t="n">
+      <c r="D5" s="322" t="n">
         <v>0.44</v>
       </c>
-      <c r="E5" s="320" t="n">
+      <c r="E5" s="323" t="n">
         <v>0.31</v>
       </c>
-      <c r="F5" s="321" t="n">
+      <c r="F5" s="324" t="n">
         <v>0.27</v>
       </c>
-      <c r="G5" s="321" t="n">
+      <c r="G5" s="324" t="n">
         <v>0.22</v>
       </c>
-      <c r="H5" s="322" t="n">
+      <c r="H5" s="325" t="n">
         <v>0.19</v>
       </c>
-      <c r="I5" s="322" t="n">
+      <c r="I5" s="325" t="n">
         <v>0.17</v>
       </c>
-      <c r="J5" s="322" t="n">
+      <c r="J5" s="325" t="n">
         <v>0.15</v>
       </c>
-      <c r="K5" s="322" t="n">
+      <c r="K5" s="325" t="n">
         <v>0.14</v>
       </c>
-      <c r="L5" s="322" t="n">
+      <c r="L5" s="325" t="n">
         <v>0.13</v>
       </c>
-      <c r="M5" s="322" t="n">
+      <c r="M5" s="325" t="n">
         <v>0.12</v>
       </c>
-      <c r="N5" s="322" t="n">
+      <c r="N5" s="325" t="n">
         <v>0.11</v>
       </c>
-      <c r="O5" s="322" t="n">
+      <c r="O5" s="325" t="n">
         <v>0.1</v>
       </c>
     </row>
     <row r="6" ht="18" customHeight="1">
-      <c r="A6" s="316" t="inlineStr">
+      <c r="A6" s="319" t="inlineStr">
         <is>
           <t>Dec-20</t>
         </is>
       </c>
-      <c r="B6" s="317" t="n">
+      <c r="B6" s="320" t="n">
         <v>3200</v>
       </c>
-      <c r="C6" s="318" t="n">
+      <c r="C6" s="321" t="n">
         <v>1</v>
       </c>
-      <c r="D6" s="319" t="n">
+      <c r="D6" s="322" t="n">
         <v>0.43</v>
       </c>
-      <c r="E6" s="320" t="n">
+      <c r="E6" s="323" t="n">
         <v>0.3</v>
       </c>
-      <c r="F6" s="321" t="n">
+      <c r="F6" s="324" t="n">
         <v>0.26</v>
       </c>
-      <c r="G6" s="321" t="n">
+      <c r="G6" s="324" t="n">
         <v>0.21</v>
       </c>
-      <c r="H6" s="322" t="n">
+      <c r="H6" s="325" t="n">
         <v>0.18</v>
       </c>
-      <c r="I6" s="322" t="n">
+      <c r="I6" s="325" t="n">
         <v>0.16</v>
       </c>
-      <c r="J6" s="322" t="n">
+      <c r="J6" s="325" t="n">
         <v>0.14</v>
       </c>
-      <c r="K6" s="322" t="n">
+      <c r="K6" s="325" t="n">
         <v>0.13</v>
       </c>
-      <c r="L6" s="322" t="n">
+      <c r="L6" s="325" t="n">
         <v>0.12</v>
       </c>
-      <c r="M6" s="322" t="n">
+      <c r="M6" s="325" t="n">
         <v>0.11</v>
       </c>
-      <c r="N6" s="322" t="n">
+      <c r="N6" s="325" t="n">
         <v>0.1</v>
       </c>
-      <c r="O6" s="323" t="n"/>
+      <c r="O6" s="326" t="n"/>
     </row>
     <row r="7" ht="18" customHeight="1">
-      <c r="A7" s="316" t="inlineStr">
+      <c r="A7" s="319" t="inlineStr">
         <is>
           <t>Jan-21</t>
         </is>
       </c>
-      <c r="B7" s="317" t="n">
+      <c r="B7" s="320" t="n">
         <v>2900</v>
       </c>
-      <c r="C7" s="318" t="n">
+      <c r="C7" s="321" t="n">
         <v>1</v>
       </c>
-      <c r="D7" s="319" t="n">
+      <c r="D7" s="322" t="n">
         <v>0.45</v>
       </c>
-      <c r="E7" s="320" t="n">
+      <c r="E7" s="323" t="n">
         <v>0.32</v>
       </c>
-      <c r="F7" s="321" t="n">
+      <c r="F7" s="324" t="n">
         <v>0.28</v>
       </c>
-      <c r="G7" s="321" t="n">
+      <c r="G7" s="324" t="n">
         <v>0.23</v>
       </c>
-      <c r="H7" s="321" t="n">
+      <c r="H7" s="324" t="n">
         <v>0.2</v>
       </c>
-      <c r="I7" s="322" t="n">
+      <c r="I7" s="325" t="n">
         <v>0.18</v>
       </c>
-      <c r="J7" s="322" t="n">
+      <c r="J7" s="325" t="n">
         <v>0.16</v>
       </c>
-      <c r="K7" s="322" t="n">
+      <c r="K7" s="325" t="n">
         <v>0.15</v>
       </c>
-      <c r="L7" s="322" t="n">
+      <c r="L7" s="325" t="n">
         <v>0.14</v>
       </c>
-      <c r="M7" s="322" t="n">
+      <c r="M7" s="325" t="n">
         <v>0.13</v>
       </c>
-      <c r="N7" s="323" t="n"/>
-      <c r="O7" s="323" t="n"/>
+      <c r="N7" s="326" t="n"/>
+      <c r="O7" s="326" t="n"/>
     </row>
     <row r="8" ht="18" customHeight="1">
-      <c r="A8" s="316" t="inlineStr">
+      <c r="A8" s="319" t="inlineStr">
         <is>
           <t>Feb-21</t>
         </is>
       </c>
-      <c r="B8" s="317" t="n">
+      <c r="B8" s="320" t="n">
         <v>2600</v>
       </c>
-      <c r="C8" s="318" t="n">
+      <c r="C8" s="321" t="n">
         <v>1</v>
       </c>
-      <c r="D8" s="319" t="n">
+      <c r="D8" s="322" t="n">
         <v>0.41</v>
       </c>
-      <c r="E8" s="321" t="n">
+      <c r="E8" s="324" t="n">
         <v>0.29</v>
       </c>
-      <c r="F8" s="321" t="n">
+      <c r="F8" s="324" t="n">
         <v>0.25</v>
       </c>
-      <c r="G8" s="321" t="n">
+      <c r="G8" s="324" t="n">
         <v>0.2</v>
       </c>
-      <c r="H8" s="322" t="n">
+      <c r="H8" s="325" t="n">
         <v>0.17</v>
       </c>
-      <c r="I8" s="322" t="n">
+      <c r="I8" s="325" t="n">
         <v>0.15</v>
       </c>
-      <c r="J8" s="322" t="n">
+      <c r="J8" s="325" t="n">
         <v>0.13</v>
       </c>
-      <c r="K8" s="322" t="n">
+      <c r="K8" s="325" t="n">
         <v>0.12</v>
       </c>
-      <c r="L8" s="322" t="n">
+      <c r="L8" s="325" t="n">
         <v>0.11</v>
       </c>
-      <c r="M8" s="323" t="n"/>
-      <c r="N8" s="323" t="n"/>
-      <c r="O8" s="323" t="n"/>
+      <c r="M8" s="326" t="n"/>
+      <c r="N8" s="326" t="n"/>
+      <c r="O8" s="326" t="n"/>
     </row>
     <row r="9" ht="18" customHeight="1">
-      <c r="A9" s="316" t="inlineStr">
+      <c r="A9" s="319" t="inlineStr">
         <is>
           <t>Mar-21</t>
         </is>
       </c>
-      <c r="B9" s="317" t="n">
+      <c r="B9" s="320" t="n">
         <v>3100</v>
       </c>
-      <c r="C9" s="318" t="n">
+      <c r="C9" s="321" t="n">
         <v>1</v>
       </c>
-      <c r="D9" s="319" t="n">
+      <c r="D9" s="322" t="n">
         <v>0.42</v>
       </c>
-      <c r="E9" s="320" t="n">
+      <c r="E9" s="323" t="n">
         <v>0.3</v>
       </c>
-      <c r="F9" s="321" t="n">
+      <c r="F9" s="324" t="n">
         <v>0.26</v>
       </c>
-      <c r="G9" s="321" t="n">
+      <c r="G9" s="324" t="n">
         <v>0.21</v>
       </c>
-      <c r="H9" s="322" t="n">
+      <c r="H9" s="325" t="n">
         <v>0.18</v>
       </c>
-      <c r="I9" s="322" t="n">
+      <c r="I9" s="325" t="n">
         <v>0.16</v>
       </c>
-      <c r="J9" s="322" t="n">
+      <c r="J9" s="325" t="n">
         <v>0.14</v>
       </c>
-      <c r="K9" s="322" t="n">
+      <c r="K9" s="325" t="n">
         <v>0.13</v>
       </c>
-      <c r="L9" s="323" t="n"/>
-      <c r="M9" s="323" t="n"/>
-      <c r="N9" s="323" t="n"/>
-      <c r="O9" s="323" t="n"/>
+      <c r="L9" s="326" t="n"/>
+      <c r="M9" s="326" t="n"/>
+      <c r="N9" s="326" t="n"/>
+      <c r="O9" s="326" t="n"/>
     </row>
     <row r="10" ht="18" customHeight="1">
-      <c r="A10" s="316" t="inlineStr">
+      <c r="A10" s="319" t="inlineStr">
         <is>
           <t>Apr-21</t>
         </is>
       </c>
-      <c r="B10" s="317" t="n">
+      <c r="B10" s="320" t="n">
         <v>2800</v>
       </c>
-      <c r="C10" s="318" t="n">
+      <c r="C10" s="321" t="n">
         <v>1</v>
       </c>
-      <c r="D10" s="319" t="n">
+      <c r="D10" s="322" t="n">
         <v>0.4</v>
       </c>
-      <c r="E10" s="321" t="n">
+      <c r="E10" s="324" t="n">
         <v>0.28</v>
       </c>
-      <c r="F10" s="321" t="n">
+      <c r="F10" s="324" t="n">
         <v>0.24</v>
       </c>
-      <c r="G10" s="322" t="n">
+      <c r="G10" s="325" t="n">
         <v>0.19</v>
       </c>
-      <c r="H10" s="322" t="n">
+      <c r="H10" s="325" t="n">
         <v>0.17</v>
       </c>
-      <c r="I10" s="322" t="n">
+      <c r="I10" s="325" t="n">
         <v>0.15</v>
       </c>
-      <c r="J10" s="322" t="n">
+      <c r="J10" s="325" t="n">
         <v>0.13</v>
       </c>
-      <c r="K10" s="323" t="n"/>
-      <c r="L10" s="323" t="n"/>
-      <c r="M10" s="323" t="n"/>
-      <c r="N10" s="323" t="n"/>
-      <c r="O10" s="323" t="n"/>
+      <c r="K10" s="326" t="n"/>
+      <c r="L10" s="326" t="n"/>
+      <c r="M10" s="326" t="n"/>
+      <c r="N10" s="326" t="n"/>
+      <c r="O10" s="326" t="n"/>
     </row>
     <row r="11" ht="18" customHeight="1">
-      <c r="A11" s="316" t="inlineStr">
+      <c r="A11" s="319" t="inlineStr">
         <is>
           <t>May-21</t>
         </is>
       </c>
-      <c r="B11" s="317" t="n">
+      <c r="B11" s="320" t="n">
         <v>3300</v>
       </c>
-      <c r="C11" s="318" t="n">
+      <c r="C11" s="321" t="n">
         <v>1</v>
       </c>
-      <c r="D11" s="319" t="n">
+      <c r="D11" s="322" t="n">
         <v>0.43</v>
       </c>
-      <c r="E11" s="320" t="n">
+      <c r="E11" s="323" t="n">
         <v>0.31</v>
       </c>
-      <c r="F11" s="321" t="n">
+      <c r="F11" s="324" t="n">
         <v>0.27</v>
       </c>
-      <c r="G11" s="321" t="n">
+      <c r="G11" s="324" t="n">
         <v>0.22</v>
       </c>
-      <c r="H11" s="322" t="n">
+      <c r="H11" s="325" t="n">
         <v>0.19</v>
       </c>
-      <c r="I11" s="322" t="n">
+      <c r="I11" s="325" t="n">
         <v>0.17</v>
       </c>
-      <c r="J11" s="323" t="n"/>
-      <c r="K11" s="323" t="n"/>
-      <c r="L11" s="323" t="n"/>
-      <c r="M11" s="323" t="n"/>
-      <c r="N11" s="323" t="n"/>
-      <c r="O11" s="323" t="n"/>
+      <c r="J11" s="326" t="n"/>
+      <c r="K11" s="326" t="n"/>
+      <c r="L11" s="326" t="n"/>
+      <c r="M11" s="326" t="n"/>
+      <c r="N11" s="326" t="n"/>
+      <c r="O11" s="326" t="n"/>
     </row>
     <row r="12" ht="18" customHeight="1">
-      <c r="A12" s="316" t="inlineStr">
+      <c r="A12" s="319" t="inlineStr">
         <is>
           <t>Jun-21</t>
         </is>
       </c>
-      <c r="B12" s="317" t="n">
+      <c r="B12" s="320" t="n">
         <v>3500</v>
       </c>
-      <c r="C12" s="318" t="n">
+      <c r="C12" s="321" t="n">
         <v>1</v>
       </c>
-      <c r="D12" s="319" t="n">
+      <c r="D12" s="322" t="n">
         <v>0.44</v>
       </c>
-      <c r="E12" s="320" t="n">
+      <c r="E12" s="323" t="n">
         <v>0.32</v>
       </c>
-      <c r="F12" s="321" t="n">
+      <c r="F12" s="324" t="n">
         <v>0.28</v>
       </c>
-      <c r="G12" s="321" t="n">
+      <c r="G12" s="324" t="n">
         <v>0.23</v>
       </c>
-      <c r="H12" s="321" t="n">
+      <c r="H12" s="324" t="n">
         <v>0.2</v>
       </c>
-      <c r="I12" s="323" t="n"/>
-      <c r="J12" s="323" t="n"/>
-      <c r="K12" s="323" t="n"/>
-      <c r="L12" s="323" t="n"/>
-      <c r="M12" s="323" t="n"/>
-      <c r="N12" s="323" t="n"/>
-      <c r="O12" s="323" t="n"/>
+      <c r="I12" s="326" t="n"/>
+      <c r="J12" s="326" t="n"/>
+      <c r="K12" s="326" t="n"/>
+      <c r="L12" s="326" t="n"/>
+      <c r="M12" s="326" t="n"/>
+      <c r="N12" s="326" t="n"/>
+      <c r="O12" s="326" t="n"/>
     </row>
     <row r="13" ht="18" customHeight="1">
-      <c r="A13" s="316" t="inlineStr">
+      <c r="A13" s="319" t="inlineStr">
         <is>
           <t>Jul-21</t>
         </is>
       </c>
-      <c r="B13" s="317" t="n">
+      <c r="B13" s="320" t="n">
         <v>2700</v>
       </c>
-      <c r="C13" s="318" t="n">
+      <c r="C13" s="321" t="n">
         <v>1</v>
       </c>
-      <c r="D13" s="319" t="n">
+      <c r="D13" s="322" t="n">
         <v>0.46</v>
       </c>
-      <c r="E13" s="320" t="n">
+      <c r="E13" s="323" t="n">
         <v>0.33</v>
       </c>
-      <c r="F13" s="321" t="n">
+      <c r="F13" s="324" t="n">
         <v>0.29</v>
       </c>
-      <c r="G13" s="321" t="n">
+      <c r="G13" s="324" t="n">
         <v>0.24</v>
       </c>
-      <c r="H13" s="323" t="n"/>
-      <c r="I13" s="323" t="n"/>
-      <c r="J13" s="323" t="n"/>
-      <c r="K13" s="323" t="n"/>
-      <c r="L13" s="323" t="n"/>
-      <c r="M13" s="323" t="n"/>
-      <c r="N13" s="323" t="n"/>
-      <c r="O13" s="323" t="n"/>
+      <c r="H13" s="326" t="n"/>
+      <c r="I13" s="326" t="n"/>
+      <c r="J13" s="326" t="n"/>
+      <c r="K13" s="326" t="n"/>
+      <c r="L13" s="326" t="n"/>
+      <c r="M13" s="326" t="n"/>
+      <c r="N13" s="326" t="n"/>
+      <c r="O13" s="326" t="n"/>
     </row>
     <row r="14" ht="18" customHeight="1">
-      <c r="A14" s="316" t="inlineStr">
+      <c r="A14" s="319" t="inlineStr">
         <is>
           <t>Aug-21</t>
         </is>
       </c>
-      <c r="B14" s="317" t="n">
+      <c r="B14" s="320" t="n">
         <v>3000</v>
       </c>
-      <c r="C14" s="318" t="n">
+      <c r="C14" s="321" t="n">
         <v>1</v>
       </c>
-      <c r="D14" s="319" t="n">
+      <c r="D14" s="322" t="n">
         <v>0.47</v>
       </c>
-      <c r="E14" s="320" t="n">
+      <c r="E14" s="323" t="n">
         <v>0.34</v>
       </c>
-      <c r="F14" s="320" t="n">
+      <c r="F14" s="323" t="n">
         <v>0.3</v>
       </c>
-      <c r="G14" s="323" t="n"/>
-      <c r="H14" s="323" t="n"/>
-      <c r="I14" s="323" t="n"/>
-      <c r="J14" s="323" t="n"/>
-      <c r="K14" s="323" t="n"/>
-      <c r="L14" s="323" t="n"/>
-      <c r="M14" s="323" t="n"/>
-      <c r="N14" s="323" t="n"/>
-      <c r="O14" s="323" t="n"/>
+      <c r="G14" s="326" t="n"/>
+      <c r="H14" s="326" t="n"/>
+      <c r="I14" s="326" t="n"/>
+      <c r="J14" s="326" t="n"/>
+      <c r="K14" s="326" t="n"/>
+      <c r="L14" s="326" t="n"/>
+      <c r="M14" s="326" t="n"/>
+      <c r="N14" s="326" t="n"/>
+      <c r="O14" s="326" t="n"/>
     </row>
     <row r="15" ht="18" customHeight="1">
-      <c r="A15" s="316" t="inlineStr">
+      <c r="A15" s="319" t="inlineStr">
         <is>
           <t>Sep-21</t>
         </is>
       </c>
-      <c r="B15" s="317" t="n">
+      <c r="B15" s="320" t="n">
         <v>2900</v>
       </c>
-      <c r="C15" s="318" t="n">
+      <c r="C15" s="321" t="n">
         <v>1</v>
       </c>
-      <c r="D15" s="319" t="n">
+      <c r="D15" s="322" t="n">
         <v>0.45</v>
       </c>
-      <c r="E15" s="320" t="n">
+      <c r="E15" s="323" t="n">
         <v>0.33</v>
       </c>
-      <c r="F15" s="323" t="n"/>
-      <c r="G15" s="323" t="n"/>
-      <c r="H15" s="323" t="n"/>
-      <c r="I15" s="323" t="n"/>
-      <c r="J15" s="323" t="n"/>
-      <c r="K15" s="323" t="n"/>
-      <c r="L15" s="323" t="n"/>
-      <c r="M15" s="323" t="n"/>
-      <c r="N15" s="323" t="n"/>
-      <c r="O15" s="323" t="n"/>
+      <c r="F15" s="326" t="n"/>
+      <c r="G15" s="326" t="n"/>
+      <c r="H15" s="326" t="n"/>
+      <c r="I15" s="326" t="n"/>
+      <c r="J15" s="326" t="n"/>
+      <c r="K15" s="326" t="n"/>
+      <c r="L15" s="326" t="n"/>
+      <c r="M15" s="326" t="n"/>
+      <c r="N15" s="326" t="n"/>
+      <c r="O15" s="326" t="n"/>
     </row>
     <row r="16" ht="18" customHeight="1">
-      <c r="A16" s="316" t="inlineStr">
+      <c r="A16" s="319" t="inlineStr">
         <is>
           <t>Oct-21</t>
         </is>
       </c>
-      <c r="B16" s="317" t="n">
+      <c r="B16" s="320" t="n">
         <v>3100</v>
       </c>
-      <c r="C16" s="318" t="n">
+      <c r="C16" s="321" t="n">
         <v>1</v>
       </c>
-      <c r="D16" s="319" t="n">
+      <c r="D16" s="322" t="n">
         <v>0.43</v>
       </c>
-      <c r="E16" s="323" t="n"/>
-      <c r="F16" s="323" t="n"/>
-      <c r="G16" s="323" t="n"/>
-      <c r="H16" s="323" t="n"/>
-      <c r="I16" s="323" t="n"/>
-      <c r="J16" s="323" t="n"/>
-      <c r="K16" s="323" t="n"/>
-      <c r="L16" s="323" t="n"/>
-      <c r="M16" s="323" t="n"/>
-      <c r="N16" s="323" t="n"/>
-      <c r="O16" s="323" t="n"/>
+      <c r="E16" s="326" t="n"/>
+      <c r="F16" s="326" t="n"/>
+      <c r="G16" s="326" t="n"/>
+      <c r="H16" s="326" t="n"/>
+      <c r="I16" s="326" t="n"/>
+      <c r="J16" s="326" t="n"/>
+      <c r="K16" s="326" t="n"/>
+      <c r="L16" s="326" t="n"/>
+      <c r="M16" s="326" t="n"/>
+      <c r="N16" s="326" t="n"/>
+      <c r="O16" s="326" t="n"/>
     </row>
     <row r="18" ht="6" customHeight="1"/>
     <row r="19" ht="16" customHeight="1">
-      <c r="A19" s="324" t="inlineStr">
-        <is>
-          <t>LEGEND:  ■ ≥40% (dark blue)   ■ ≥30% (medium blue)   ■ ≥20% (light blue)   ■ ≥10% (pale blue)   ■ &lt;10% (very pale)   ■ No data (grey)</t>
+      <c r="A19" s="327" t="inlineStr">
+        <is>
+          <t>LEGEND:  ■ ≥40% (dark amber)   ■ ≥30% (amber)   ■ ≥20% (gold)   ■ ≥10% (light gold)   ■ &lt;10% (pale yellow)   ■ No data (grey)</t>
         </is>
       </c>
     </row>
@@ -16531,14 +16588,14 @@
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
-      <c r="A1" s="325" t="inlineStr">
+      <c r="A1" s="328" t="inlineStr">
         <is>
           <t>CHANNEL ROI ANALYSIS  ·  Marketing Attribution  ·  GA4 Intelligence Hub</t>
         </is>
       </c>
     </row>
     <row r="2" ht="16" customHeight="1">
-      <c r="A2" s="326" t="inlineStr">
+      <c r="A2" s="329" t="inlineStr">
         <is>
           <t>Total Revenue: $891,480  ·  Paid Spend: $214,800  ·  Blended ROAS: 4.15x  ·  Blended CPA: $25.55</t>
         </is>
@@ -16546,69 +16603,69 @@
     </row>
     <row r="3" ht="6" customHeight="1"/>
     <row r="4" ht="22" customHeight="1">
-      <c r="A4" s="327" t="inlineStr">
+      <c r="A4" s="330" t="inlineStr">
         <is>
           <t>Channel</t>
         </is>
       </c>
-      <c r="B4" s="327" t="inlineStr">
+      <c r="B4" s="330" t="inlineStr">
         <is>
           <t>Source/Medium</t>
         </is>
       </c>
-      <c r="C4" s="327" t="inlineStr">
+      <c r="C4" s="330" t="inlineStr">
         <is>
           <t>Revenue ($)</t>
         </is>
       </c>
-      <c r="D4" s="327" t="inlineStr">
+      <c r="D4" s="330" t="inlineStr">
         <is>
           <t>Sessions</t>
         </is>
       </c>
-      <c r="E4" s="327" t="inlineStr">
+      <c r="E4" s="330" t="inlineStr">
         <is>
           <t>Txns</t>
         </is>
       </c>
-      <c r="F4" s="327" t="inlineStr">
+      <c r="F4" s="330" t="inlineStr">
         <is>
           <t>CVR %</t>
         </is>
       </c>
-      <c r="G4" s="327" t="inlineStr">
+      <c r="G4" s="330" t="inlineStr">
         <is>
           <t>Ad Spend ($)</t>
         </is>
       </c>
-      <c r="H4" s="327" t="inlineStr">
+      <c r="H4" s="330" t="inlineStr">
         <is>
           <t>ROAS</t>
         </is>
       </c>
-      <c r="I4" s="327" t="inlineStr">
+      <c r="I4" s="330" t="inlineStr">
         <is>
           <t>CPA ($)</t>
         </is>
       </c>
-      <c r="J4" s="327" t="inlineStr">
+      <c r="J4" s="330" t="inlineStr">
         <is>
           <t>% of Revenue</t>
         </is>
       </c>
     </row>
     <row r="5" ht="20" customHeight="1">
-      <c r="A5" s="328" t="inlineStr">
+      <c r="A5" s="331" t="inlineStr">
         <is>
           <t>Organic Search</t>
         </is>
       </c>
-      <c r="B5" s="329" t="inlineStr">
+      <c r="B5" s="332" t="inlineStr">
         <is>
           <t>google / organic</t>
         </is>
       </c>
-      <c r="C5" s="270" t="n">
+      <c r="C5" s="333" t="n">
         <v>298500</v>
       </c>
       <c r="D5" s="271" t="n">
@@ -16617,10 +16674,10 @@
       <c r="E5" s="271" t="n">
         <v>11070</v>
       </c>
-      <c r="F5" s="330" t="n">
+      <c r="F5" s="334" t="n">
         <v>0.0155</v>
       </c>
-      <c r="G5" s="331" t="inlineStr">
+      <c r="G5" s="335" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
@@ -16630,69 +16687,69 @@
           <t>Organic</t>
         </is>
       </c>
-      <c r="I5" s="331" t="inlineStr">
+      <c r="I5" s="335" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="J5" s="332" t="n">
+      <c r="J5" s="336" t="n">
         <v>0.3349</v>
       </c>
     </row>
     <row r="6" ht="20" customHeight="1">
-      <c r="A6" s="333" t="inlineStr">
+      <c r="A6" s="337" t="inlineStr">
         <is>
           <t>Direct</t>
         </is>
       </c>
-      <c r="B6" s="334" t="inlineStr">
+      <c r="B6" s="338" t="inlineStr">
         <is>
           <t>(direct) / (none)</t>
         </is>
       </c>
-      <c r="C6" s="335" t="n">
+      <c r="C6" s="339" t="n">
         <v>222380</v>
       </c>
-      <c r="D6" s="336" t="n">
+      <c r="D6" s="340" t="n">
         <v>398600</v>
       </c>
-      <c r="E6" s="336" t="n">
+      <c r="E6" s="340" t="n">
         <v>9820</v>
       </c>
-      <c r="F6" s="337" t="n">
+      <c r="F6" s="341" t="n">
         <v>0.0246</v>
       </c>
-      <c r="G6" s="338" t="inlineStr">
+      <c r="G6" s="342" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="H6" s="339" t="inlineStr">
+      <c r="H6" s="343" t="inlineStr">
         <is>
           <t>Organic</t>
         </is>
       </c>
-      <c r="I6" s="338" t="inlineStr">
+      <c r="I6" s="342" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="J6" s="340" t="n">
+      <c r="J6" s="344" t="n">
         <v>0.2494</v>
       </c>
     </row>
     <row r="7" ht="20" customHeight="1">
-      <c r="A7" s="328" t="inlineStr">
+      <c r="A7" s="331" t="inlineStr">
         <is>
           <t>Paid Search</t>
         </is>
       </c>
-      <c r="B7" s="329" t="inlineStr">
+      <c r="B7" s="332" t="inlineStr">
         <is>
           <t>google / cpc</t>
         </is>
       </c>
-      <c r="C7" s="270" t="n">
+      <c r="C7" s="333" t="n">
         <v>178400</v>
       </c>
       <c r="D7" s="271" t="n">
@@ -16701,13 +16758,13 @@
       <c r="E7" s="271" t="n">
         <v>7920</v>
       </c>
-      <c r="F7" s="330" t="n">
+      <c r="F7" s="334" t="n">
         <v>0.0203</v>
       </c>
-      <c r="G7" s="341" t="n">
+      <c r="G7" s="345" t="n">
         <v>102000</v>
       </c>
-      <c r="H7" s="288" t="inlineStr">
+      <c r="H7" s="346" t="inlineStr">
         <is>
           <t>1.75x</t>
         </is>
@@ -16715,60 +16772,60 @@
       <c r="I7" s="272" t="n">
         <v>12.88</v>
       </c>
-      <c r="J7" s="332" t="n">
+      <c r="J7" s="336" t="n">
         <v>0.2001</v>
       </c>
     </row>
     <row r="8" ht="20" customHeight="1">
-      <c r="A8" s="333" t="inlineStr">
+      <c r="A8" s="337" t="inlineStr">
         <is>
           <t>Email</t>
         </is>
       </c>
-      <c r="B8" s="334" t="inlineStr">
+      <c r="B8" s="338" t="inlineStr">
         <is>
           <t>newsletter / email</t>
         </is>
       </c>
-      <c r="C8" s="335" t="n">
+      <c r="C8" s="339" t="n">
         <v>133600</v>
       </c>
-      <c r="D8" s="336" t="n">
+      <c r="D8" s="340" t="n">
         <v>198200</v>
       </c>
-      <c r="E8" s="336" t="n">
+      <c r="E8" s="340" t="n">
         <v>4920</v>
       </c>
-      <c r="F8" s="337" t="n">
+      <c r="F8" s="341" t="n">
         <v>0.0248</v>
       </c>
-      <c r="G8" s="342" t="n">
+      <c r="G8" s="347" t="n">
         <v>62400</v>
       </c>
-      <c r="H8" s="343" t="inlineStr">
+      <c r="H8" s="348" t="inlineStr">
         <is>
           <t>2.14x</t>
         </is>
       </c>
-      <c r="I8" s="344" t="n">
+      <c r="I8" s="349" t="n">
         <v>12.68</v>
       </c>
-      <c r="J8" s="340" t="n">
+      <c r="J8" s="344" t="n">
         <v>0.1498</v>
       </c>
     </row>
     <row r="9" ht="20" customHeight="1">
-      <c r="A9" s="328" t="inlineStr">
+      <c r="A9" s="331" t="inlineStr">
         <is>
           <t>Social</t>
         </is>
       </c>
-      <c r="B9" s="329" t="inlineStr">
+      <c r="B9" s="332" t="inlineStr">
         <is>
           <t>facebook / social</t>
         </is>
       </c>
-      <c r="C9" s="270" t="n">
+      <c r="C9" s="333" t="n">
         <v>44600</v>
       </c>
       <c r="D9" s="271" t="n">
@@ -16777,13 +16834,13 @@
       <c r="E9" s="271" t="n">
         <v>1020</v>
       </c>
-      <c r="F9" s="330" t="n">
+      <c r="F9" s="334" t="n">
         <v>0.0075</v>
       </c>
-      <c r="G9" s="341" t="n">
+      <c r="G9" s="345" t="n">
         <v>38400</v>
       </c>
-      <c r="H9" s="288" t="inlineStr">
+      <c r="H9" s="346" t="inlineStr">
         <is>
           <t>1.16x</t>
         </is>
@@ -16791,60 +16848,60 @@
       <c r="I9" s="272" t="n">
         <v>37.65</v>
       </c>
-      <c r="J9" s="332" t="n">
+      <c r="J9" s="336" t="n">
         <v>0.05</v>
       </c>
     </row>
     <row r="10" ht="20" customHeight="1">
-      <c r="A10" s="333" t="inlineStr">
+      <c r="A10" s="337" t="inlineStr">
         <is>
           <t>Referral</t>
         </is>
       </c>
-      <c r="B10" s="334" t="inlineStr">
+      <c r="B10" s="338" t="inlineStr">
         <is>
           <t>partners / referral</t>
         </is>
       </c>
-      <c r="C10" s="335" t="n">
+      <c r="C10" s="339" t="n">
         <v>13310</v>
       </c>
-      <c r="D10" s="336" t="n">
+      <c r="D10" s="340" t="n">
         <v>54600</v>
       </c>
-      <c r="E10" s="336" t="n">
+      <c r="E10" s="340" t="n">
         <v>108</v>
       </c>
-      <c r="F10" s="337" t="n">
+      <c r="F10" s="341" t="n">
         <v>0.002</v>
       </c>
-      <c r="G10" s="342" t="n">
+      <c r="G10" s="347" t="n">
         <v>12000</v>
       </c>
-      <c r="H10" s="345" t="inlineStr">
+      <c r="H10" s="350" t="inlineStr">
         <is>
           <t>1.11x</t>
         </is>
       </c>
-      <c r="I10" s="344" t="n">
+      <c r="I10" s="349" t="n">
         <v>111.11</v>
       </c>
-      <c r="J10" s="340" t="n">
+      <c r="J10" s="344" t="n">
         <v>0.0149</v>
       </c>
     </row>
     <row r="11" ht="20" customHeight="1">
-      <c r="A11" s="328" t="inlineStr">
+      <c r="A11" s="331" t="inlineStr">
         <is>
           <t>Display</t>
         </is>
       </c>
-      <c r="B11" s="329" t="inlineStr">
+      <c r="B11" s="332" t="inlineStr">
         <is>
           <t>google / display</t>
         </is>
       </c>
-      <c r="C11" s="270" t="n">
+      <c r="C11" s="333" t="n">
         <v>690</v>
       </c>
       <c r="D11" s="271" t="n">
@@ -16853,10 +16910,10 @@
       <c r="E11" s="271" t="n">
         <v>32</v>
       </c>
-      <c r="F11" s="330" t="n">
+      <c r="F11" s="334" t="n">
         <v>0.0133</v>
       </c>
-      <c r="G11" s="331" t="inlineStr">
+      <c r="G11" s="335" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
@@ -16866,36 +16923,36 @@
           <t>Organic</t>
         </is>
       </c>
-      <c r="I11" s="331" t="inlineStr">
+      <c r="I11" s="335" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="J11" s="332" t="n">
+      <c r="J11" s="336" t="n">
         <v>0.0008</v>
       </c>
     </row>
     <row r="12" ht="22" customHeight="1">
-      <c r="A12" s="346" t="inlineStr">
+      <c r="A12" s="351" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B12" s="347" t="n"/>
-      <c r="C12" s="348" t="n">
+      <c r="B12" s="352" t="n"/>
+      <c r="C12" s="353" t="n">
         <v>891480</v>
       </c>
-      <c r="D12" s="349" t="n">
+      <c r="D12" s="354" t="n">
         <v>1892200</v>
       </c>
-      <c r="E12" s="349" t="n">
+      <c r="E12" s="354" t="n">
         <v>34890</v>
       </c>
-      <c r="F12" s="347" t="n"/>
-      <c r="G12" s="347" t="n"/>
-      <c r="H12" s="347" t="n"/>
-      <c r="I12" s="347" t="n"/>
-      <c r="J12" s="347" t="n"/>
+      <c r="F12" s="352" t="n"/>
+      <c r="G12" s="352" t="n"/>
+      <c r="H12" s="352" t="n"/>
+      <c r="I12" s="352" t="n"/>
+      <c r="J12" s="352" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -16930,14 +16987,14 @@
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
-      <c r="A1" s="350" t="inlineStr">
+      <c r="A1" s="355" t="inlineStr">
         <is>
           <t>RFM SEGMENTATION  ·  Recency · Frequency · Monetary  ·  GA4 Intelligence Hub</t>
         </is>
       </c>
     </row>
     <row r="2" ht="16" customHeight="1">
-      <c r="A2" s="351" t="inlineStr">
+      <c r="A2" s="356" t="inlineStr">
         <is>
           <t>Scoring: Recency 1-5 (5=purchased recently)  ·  Frequency 1-5 (5=most orders)  ·  Monetary 1-5 (5=highest spend)  ·  RFM Score = R+F+M (max 15)</t>
         </is>
@@ -16945,69 +17002,69 @@
     </row>
     <row r="3" ht="6" customHeight="1"/>
     <row r="4" ht="22" customHeight="1">
-      <c r="A4" s="352" t="inlineStr">
+      <c r="A4" s="357" t="inlineStr">
         <is>
           <t>Customer ID</t>
         </is>
       </c>
-      <c r="B4" s="352" t="inlineStr">
+      <c r="B4" s="357" t="inlineStr">
         <is>
           <t>Tier</t>
         </is>
       </c>
-      <c r="C4" s="352" t="inlineStr">
+      <c r="C4" s="357" t="inlineStr">
         <is>
           <t>Days Since</t>
         </is>
       </c>
-      <c r="D4" s="352" t="inlineStr">
+      <c r="D4" s="357" t="inlineStr">
         <is>
           <t>Recency (R)</t>
         </is>
       </c>
-      <c r="E4" s="352" t="inlineStr">
+      <c r="E4" s="357" t="inlineStr">
         <is>
           <t>Orders</t>
         </is>
       </c>
-      <c r="F4" s="352" t="inlineStr">
+      <c r="F4" s="357" t="inlineStr">
         <is>
           <t>Frequency (F)</t>
         </is>
       </c>
-      <c r="G4" s="352" t="inlineStr">
+      <c r="G4" s="357" t="inlineStr">
         <is>
           <t>Total Spend</t>
         </is>
       </c>
-      <c r="H4" s="352" t="inlineStr">
+      <c r="H4" s="357" t="inlineStr">
         <is>
           <t>Monetary (M)</t>
         </is>
       </c>
-      <c r="I4" s="352" t="inlineStr">
+      <c r="I4" s="357" t="inlineStr">
         <is>
           <t>RFM Score</t>
         </is>
       </c>
-      <c r="J4" s="352" t="inlineStr">
+      <c r="J4" s="357" t="inlineStr">
         <is>
           <t>Segment</t>
         </is>
       </c>
-      <c r="K4" s="352" t="inlineStr">
+      <c r="K4" s="357" t="inlineStr">
         <is>
           <t>Action</t>
         </is>
       </c>
     </row>
     <row r="5" ht="18" customHeight="1">
-      <c r="A5" s="353" t="inlineStr">
+      <c r="A5" s="358" t="inlineStr">
         <is>
           <t>C-001</t>
         </is>
       </c>
-      <c r="B5" s="354" t="inlineStr">
+      <c r="B5" s="359" t="inlineStr">
         <is>
           <t>Platinum</t>
         </is>
@@ -17015,25 +17072,25 @@
       <c r="C5" s="271" t="n">
         <v>3</v>
       </c>
-      <c r="D5" s="355" t="n">
+      <c r="D5" s="360" t="n">
         <v>5</v>
       </c>
       <c r="E5" s="271" t="n">
         <v>22</v>
       </c>
-      <c r="F5" s="356" t="n">
+      <c r="F5" s="361" t="n">
         <v>5</v>
       </c>
-      <c r="G5" s="357" t="n">
+      <c r="G5" s="362" t="n">
         <v>892.4</v>
       </c>
-      <c r="H5" s="358" t="n">
+      <c r="H5" s="363" t="n">
         <v>5</v>
       </c>
-      <c r="I5" s="355" t="n">
+      <c r="I5" s="364" t="n">
         <v>15</v>
       </c>
-      <c r="J5" s="354" t="inlineStr">
+      <c r="J5" s="359" t="inlineStr">
         <is>
           <t>Champion</t>
         </is>
@@ -17045,55 +17102,55 @@
       </c>
     </row>
     <row r="6" ht="18" customHeight="1">
-      <c r="A6" s="359" t="inlineStr">
+      <c r="A6" s="365" t="inlineStr">
         <is>
           <t>C-002</t>
         </is>
       </c>
-      <c r="B6" s="354" t="inlineStr">
+      <c r="B6" s="359" t="inlineStr">
         <is>
           <t>Platinum</t>
         </is>
       </c>
-      <c r="C6" s="360" t="n">
+      <c r="C6" s="366" t="n">
         <v>5</v>
       </c>
-      <c r="D6" s="355" t="n">
+      <c r="D6" s="360" t="n">
         <v>5</v>
       </c>
-      <c r="E6" s="360" t="n">
+      <c r="E6" s="366" t="n">
         <v>18</v>
       </c>
-      <c r="F6" s="356" t="n">
+      <c r="F6" s="361" t="n">
         <v>5</v>
       </c>
-      <c r="G6" s="361" t="n">
+      <c r="G6" s="367" t="n">
         <v>748.62</v>
       </c>
-      <c r="H6" s="358" t="n">
+      <c r="H6" s="363" t="n">
         <v>5</v>
       </c>
-      <c r="I6" s="355" t="n">
+      <c r="I6" s="364" t="n">
         <v>15</v>
       </c>
-      <c r="J6" s="354" t="inlineStr">
+      <c r="J6" s="359" t="inlineStr">
         <is>
           <t>Champion</t>
         </is>
       </c>
-      <c r="K6" s="362" t="inlineStr">
+      <c r="K6" s="368" t="inlineStr">
         <is>
           <t>Exclusive preview access</t>
         </is>
       </c>
     </row>
     <row r="7" ht="18" customHeight="1">
-      <c r="A7" s="353" t="inlineStr">
+      <c r="A7" s="358" t="inlineStr">
         <is>
           <t>C-003</t>
         </is>
       </c>
-      <c r="B7" s="354" t="inlineStr">
+      <c r="B7" s="359" t="inlineStr">
         <is>
           <t>Platinum</t>
         </is>
@@ -17101,25 +17158,25 @@
       <c r="C7" s="271" t="n">
         <v>7</v>
       </c>
-      <c r="D7" s="355" t="n">
+      <c r="D7" s="360" t="n">
         <v>5</v>
       </c>
       <c r="E7" s="271" t="n">
         <v>16</v>
       </c>
-      <c r="F7" s="356" t="n">
+      <c r="F7" s="361" t="n">
         <v>5</v>
       </c>
-      <c r="G7" s="357" t="n">
+      <c r="G7" s="362" t="n">
         <v>674.91</v>
       </c>
-      <c r="H7" s="358" t="n">
+      <c r="H7" s="363" t="n">
         <v>5</v>
       </c>
-      <c r="I7" s="355" t="n">
+      <c r="I7" s="364" t="n">
         <v>15</v>
       </c>
-      <c r="J7" s="354" t="inlineStr">
+      <c r="J7" s="359" t="inlineStr">
         <is>
           <t>Champion</t>
         </is>
@@ -17131,55 +17188,55 @@
       </c>
     </row>
     <row r="8" ht="18" customHeight="1">
-      <c r="A8" s="359" t="inlineStr">
+      <c r="A8" s="365" t="inlineStr">
         <is>
           <t>C-004</t>
         </is>
       </c>
-      <c r="B8" s="354" t="inlineStr">
+      <c r="B8" s="359" t="inlineStr">
         <is>
           <t>Platinum</t>
         </is>
       </c>
-      <c r="C8" s="360" t="n">
+      <c r="C8" s="366" t="n">
         <v>4</v>
       </c>
-      <c r="D8" s="355" t="n">
+      <c r="D8" s="360" t="n">
         <v>5</v>
       </c>
-      <c r="E8" s="360" t="n">
+      <c r="E8" s="366" t="n">
         <v>14</v>
       </c>
-      <c r="F8" s="363" t="n">
+      <c r="F8" s="369" t="n">
         <v>4</v>
       </c>
-      <c r="G8" s="361" t="n">
+      <c r="G8" s="367" t="n">
         <v>589.2</v>
       </c>
-      <c r="H8" s="358" t="n">
+      <c r="H8" s="363" t="n">
         <v>5</v>
       </c>
-      <c r="I8" s="355" t="n">
+      <c r="I8" s="364" t="n">
         <v>14</v>
       </c>
-      <c r="J8" s="354" t="inlineStr">
+      <c r="J8" s="359" t="inlineStr">
         <is>
           <t>Champion</t>
         </is>
       </c>
-      <c r="K8" s="362" t="inlineStr">
+      <c r="K8" s="368" t="inlineStr">
         <is>
           <t>Co-creation opportunity</t>
         </is>
       </c>
     </row>
     <row r="9" ht="18" customHeight="1">
-      <c r="A9" s="353" t="inlineStr">
+      <c r="A9" s="358" t="inlineStr">
         <is>
           <t>C-005</t>
         </is>
       </c>
-      <c r="B9" s="354" t="inlineStr">
+      <c r="B9" s="359" t="inlineStr">
         <is>
           <t>Platinum</t>
         </is>
@@ -17187,25 +17244,25 @@
       <c r="C9" s="271" t="n">
         <v>8</v>
       </c>
-      <c r="D9" s="364" t="n">
+      <c r="D9" s="370" t="n">
         <v>4</v>
       </c>
       <c r="E9" s="271" t="n">
         <v>12</v>
       </c>
-      <c r="F9" s="363" t="n">
+      <c r="F9" s="369" t="n">
         <v>4</v>
       </c>
-      <c r="G9" s="357" t="n">
+      <c r="G9" s="362" t="n">
         <v>512.8</v>
       </c>
-      <c r="H9" s="358" t="n">
+      <c r="H9" s="363" t="n">
         <v>5</v>
       </c>
-      <c r="I9" s="355" t="n">
+      <c r="I9" s="364" t="n">
         <v>13</v>
       </c>
-      <c r="J9" s="354" t="inlineStr">
+      <c r="J9" s="359" t="inlineStr">
         <is>
           <t>Champion</t>
         </is>
@@ -17217,55 +17274,55 @@
       </c>
     </row>
     <row r="10" ht="18" customHeight="1">
-      <c r="A10" s="359" t="inlineStr">
+      <c r="A10" s="365" t="inlineStr">
         <is>
           <t>C-006</t>
         </is>
       </c>
-      <c r="B10" s="365" t="inlineStr">
+      <c r="B10" s="371" t="inlineStr">
         <is>
           <t>Gold</t>
         </is>
       </c>
-      <c r="C10" s="360" t="n">
+      <c r="C10" s="366" t="n">
         <v>14</v>
       </c>
-      <c r="D10" s="364" t="n">
+      <c r="D10" s="370" t="n">
         <v>4</v>
       </c>
-      <c r="E10" s="360" t="n">
+      <c r="E10" s="366" t="n">
         <v>10</v>
       </c>
-      <c r="F10" s="363" t="n">
+      <c r="F10" s="369" t="n">
         <v>4</v>
       </c>
-      <c r="G10" s="361" t="n">
+      <c r="G10" s="367" t="n">
         <v>418.76</v>
       </c>
-      <c r="H10" s="366" t="n">
+      <c r="H10" s="372" t="n">
         <v>4</v>
       </c>
-      <c r="I10" s="364" t="n">
+      <c r="I10" s="370" t="n">
         <v>12</v>
       </c>
-      <c r="J10" s="365" t="inlineStr">
+      <c r="J10" s="371" t="inlineStr">
         <is>
           <t>Loyal</t>
         </is>
       </c>
-      <c r="K10" s="362" t="inlineStr">
+      <c r="K10" s="368" t="inlineStr">
         <is>
           <t>Referral programme</t>
         </is>
       </c>
     </row>
     <row r="11" ht="18" customHeight="1">
-      <c r="A11" s="353" t="inlineStr">
+      <c r="A11" s="358" t="inlineStr">
         <is>
           <t>C-007</t>
         </is>
       </c>
-      <c r="B11" s="365" t="inlineStr">
+      <c r="B11" s="371" t="inlineStr">
         <is>
           <t>Gold</t>
         </is>
@@ -17273,25 +17330,25 @@
       <c r="C11" s="271" t="n">
         <v>19</v>
       </c>
-      <c r="D11" s="364" t="n">
+      <c r="D11" s="370" t="n">
         <v>4</v>
       </c>
       <c r="E11" s="271" t="n">
         <v>9</v>
       </c>
-      <c r="F11" s="363" t="n">
+      <c r="F11" s="369" t="n">
         <v>4</v>
       </c>
-      <c r="G11" s="357" t="n">
+      <c r="G11" s="362" t="n">
         <v>362.91</v>
       </c>
-      <c r="H11" s="366" t="n">
+      <c r="H11" s="372" t="n">
         <v>4</v>
       </c>
-      <c r="I11" s="364" t="n">
+      <c r="I11" s="370" t="n">
         <v>12</v>
       </c>
-      <c r="J11" s="365" t="inlineStr">
+      <c r="J11" s="371" t="inlineStr">
         <is>
           <t>Loyal</t>
         </is>
@@ -17303,55 +17360,55 @@
       </c>
     </row>
     <row r="12" ht="18" customHeight="1">
-      <c r="A12" s="359" t="inlineStr">
+      <c r="A12" s="365" t="inlineStr">
         <is>
           <t>C-008</t>
         </is>
       </c>
-      <c r="B12" s="365" t="inlineStr">
+      <c r="B12" s="371" t="inlineStr">
         <is>
           <t>Gold</t>
         </is>
       </c>
-      <c r="C12" s="360" t="n">
+      <c r="C12" s="366" t="n">
         <v>22</v>
       </c>
-      <c r="D12" s="367" t="n">
+      <c r="D12" s="373" t="n">
         <v>3</v>
       </c>
-      <c r="E12" s="360" t="n">
+      <c r="E12" s="366" t="n">
         <v>8</v>
       </c>
-      <c r="F12" s="363" t="n">
+      <c r="F12" s="369" t="n">
         <v>4</v>
       </c>
-      <c r="G12" s="361" t="n">
+      <c r="G12" s="367" t="n">
         <v>319.8</v>
       </c>
-      <c r="H12" s="366" t="n">
+      <c r="H12" s="372" t="n">
         <v>4</v>
       </c>
-      <c r="I12" s="364" t="n">
+      <c r="I12" s="370" t="n">
         <v>11</v>
       </c>
-      <c r="J12" s="365" t="inlineStr">
+      <c r="J12" s="371" t="inlineStr">
         <is>
           <t>Loyal</t>
         </is>
       </c>
-      <c r="K12" s="362" t="inlineStr">
+      <c r="K12" s="368" t="inlineStr">
         <is>
           <t>Seasonal bundle offer</t>
         </is>
       </c>
     </row>
     <row r="13" ht="18" customHeight="1">
-      <c r="A13" s="353" t="inlineStr">
+      <c r="A13" s="358" t="inlineStr">
         <is>
           <t>C-009</t>
         </is>
       </c>
-      <c r="B13" s="365" t="inlineStr">
+      <c r="B13" s="371" t="inlineStr">
         <is>
           <t>Gold</t>
         </is>
@@ -17359,25 +17416,25 @@
       <c r="C13" s="271" t="n">
         <v>25</v>
       </c>
-      <c r="D13" s="367" t="n">
+      <c r="D13" s="373" t="n">
         <v>3</v>
       </c>
       <c r="E13" s="271" t="n">
         <v>8</v>
       </c>
-      <c r="F13" s="363" t="n">
+      <c r="F13" s="369" t="n">
         <v>4</v>
       </c>
-      <c r="G13" s="357" t="n">
+      <c r="G13" s="362" t="n">
         <v>298.7</v>
       </c>
-      <c r="H13" s="366" t="n">
+      <c r="H13" s="372" t="n">
         <v>4</v>
       </c>
-      <c r="I13" s="364" t="n">
+      <c r="I13" s="370" t="n">
         <v>11</v>
       </c>
-      <c r="J13" s="365" t="inlineStr">
+      <c r="J13" s="371" t="inlineStr">
         <is>
           <t>Loyal</t>
         </is>
@@ -17389,55 +17446,55 @@
       </c>
     </row>
     <row r="14" ht="18" customHeight="1">
-      <c r="A14" s="359" t="inlineStr">
+      <c r="A14" s="365" t="inlineStr">
         <is>
           <t>C-010</t>
         </is>
       </c>
-      <c r="B14" s="365" t="inlineStr">
+      <c r="B14" s="371" t="inlineStr">
         <is>
           <t>Gold</t>
         </is>
       </c>
-      <c r="C14" s="360" t="n">
+      <c r="C14" s="366" t="n">
         <v>28</v>
       </c>
-      <c r="D14" s="367" t="n">
+      <c r="D14" s="373" t="n">
         <v>3</v>
       </c>
-      <c r="E14" s="360" t="n">
+      <c r="E14" s="366" t="n">
         <v>7</v>
       </c>
-      <c r="F14" s="368" t="n">
+      <c r="F14" s="374" t="n">
         <v>3</v>
       </c>
-      <c r="G14" s="361" t="n">
+      <c r="G14" s="367" t="n">
         <v>268.5</v>
       </c>
-      <c r="H14" s="366" t="n">
+      <c r="H14" s="372" t="n">
         <v>4</v>
       </c>
-      <c r="I14" s="364" t="n">
+      <c r="I14" s="370" t="n">
         <v>10</v>
       </c>
-      <c r="J14" s="365" t="inlineStr">
+      <c r="J14" s="371" t="inlineStr">
         <is>
           <t>Loyal</t>
         </is>
       </c>
-      <c r="K14" s="362" t="inlineStr">
+      <c r="K14" s="368" t="inlineStr">
         <is>
           <t>Upsell campaign</t>
         </is>
       </c>
     </row>
     <row r="15" ht="18" customHeight="1">
-      <c r="A15" s="353" t="inlineStr">
+      <c r="A15" s="358" t="inlineStr">
         <is>
           <t>C-011</t>
         </is>
       </c>
-      <c r="B15" s="365" t="inlineStr">
+      <c r="B15" s="371" t="inlineStr">
         <is>
           <t>Gold</t>
         </is>
@@ -17445,25 +17502,25 @@
       <c r="C15" s="271" t="n">
         <v>31</v>
       </c>
-      <c r="D15" s="367" t="n">
+      <c r="D15" s="373" t="n">
         <v>3</v>
       </c>
       <c r="E15" s="271" t="n">
         <v>7</v>
       </c>
-      <c r="F15" s="368" t="n">
+      <c r="F15" s="374" t="n">
         <v>3</v>
       </c>
-      <c r="G15" s="357" t="n">
+      <c r="G15" s="362" t="n">
         <v>248.4</v>
       </c>
-      <c r="H15" s="369" t="n">
+      <c r="H15" s="375" t="n">
         <v>3</v>
       </c>
-      <c r="I15" s="370" t="n">
+      <c r="I15" s="376" t="n">
         <v>9</v>
       </c>
-      <c r="J15" s="365" t="inlineStr">
+      <c r="J15" s="371" t="inlineStr">
         <is>
           <t>Loyal</t>
         </is>
@@ -17475,55 +17532,55 @@
       </c>
     </row>
     <row r="16" ht="18" customHeight="1">
-      <c r="A16" s="359" t="inlineStr">
+      <c r="A16" s="365" t="inlineStr">
         <is>
           <t>C-012</t>
         </is>
       </c>
-      <c r="B16" s="365" t="inlineStr">
+      <c r="B16" s="371" t="inlineStr">
         <is>
           <t>Gold</t>
         </is>
       </c>
-      <c r="C16" s="360" t="n">
+      <c r="C16" s="366" t="n">
         <v>35</v>
       </c>
-      <c r="D16" s="367" t="n">
+      <c r="D16" s="373" t="n">
         <v>3</v>
       </c>
-      <c r="E16" s="360" t="n">
+      <c r="E16" s="366" t="n">
         <v>6</v>
       </c>
-      <c r="F16" s="368" t="n">
+      <c r="F16" s="374" t="n">
         <v>3</v>
       </c>
-      <c r="G16" s="361" t="n">
+      <c r="G16" s="367" t="n">
         <v>224.92</v>
       </c>
-      <c r="H16" s="369" t="n">
+      <c r="H16" s="375" t="n">
         <v>3</v>
       </c>
-      <c r="I16" s="370" t="n">
+      <c r="I16" s="376" t="n">
         <v>9</v>
       </c>
-      <c r="J16" s="365" t="inlineStr">
+      <c r="J16" s="371" t="inlineStr">
         <is>
           <t>Loyal</t>
         </is>
       </c>
-      <c r="K16" s="362" t="inlineStr">
+      <c r="K16" s="368" t="inlineStr">
         <is>
           <t>Seasonal discount</t>
         </is>
       </c>
     </row>
     <row r="17" ht="18" customHeight="1">
-      <c r="A17" s="353" t="inlineStr">
+      <c r="A17" s="358" t="inlineStr">
         <is>
           <t>C-013</t>
         </is>
       </c>
-      <c r="B17" s="365" t="inlineStr">
+      <c r="B17" s="371" t="inlineStr">
         <is>
           <t>Gold</t>
         </is>
@@ -17531,25 +17588,25 @@
       <c r="C17" s="271" t="n">
         <v>38</v>
       </c>
-      <c r="D17" s="367" t="n">
+      <c r="D17" s="373" t="n">
         <v>3</v>
       </c>
       <c r="E17" s="271" t="n">
         <v>6</v>
       </c>
-      <c r="F17" s="368" t="n">
+      <c r="F17" s="374" t="n">
         <v>3</v>
       </c>
-      <c r="G17" s="357" t="n">
+      <c r="G17" s="362" t="n">
         <v>218.47</v>
       </c>
-      <c r="H17" s="369" t="n">
+      <c r="H17" s="375" t="n">
         <v>3</v>
       </c>
-      <c r="I17" s="370" t="n">
+      <c r="I17" s="376" t="n">
         <v>9</v>
       </c>
-      <c r="J17" s="365" t="inlineStr">
+      <c r="J17" s="371" t="inlineStr">
         <is>
           <t>Loyal</t>
         </is>
@@ -17561,55 +17618,55 @@
       </c>
     </row>
     <row r="18" ht="18" customHeight="1">
-      <c r="A18" s="359" t="inlineStr">
+      <c r="A18" s="365" t="inlineStr">
         <is>
           <t>C-014</t>
         </is>
       </c>
-      <c r="B18" s="371" t="inlineStr">
+      <c r="B18" s="377" t="inlineStr">
         <is>
           <t>Silver</t>
         </is>
       </c>
-      <c r="C18" s="360" t="n">
+      <c r="C18" s="366" t="n">
         <v>41</v>
       </c>
-      <c r="D18" s="367" t="n">
+      <c r="D18" s="373" t="n">
         <v>3</v>
       </c>
-      <c r="E18" s="360" t="n">
+      <c r="E18" s="366" t="n">
         <v>5</v>
       </c>
-      <c r="F18" s="368" t="n">
+      <c r="F18" s="374" t="n">
         <v>3</v>
       </c>
-      <c r="G18" s="361" t="n">
+      <c r="G18" s="367" t="n">
         <v>189.3</v>
       </c>
-      <c r="H18" s="369" t="n">
+      <c r="H18" s="375" t="n">
         <v>3</v>
       </c>
-      <c r="I18" s="370" t="n">
+      <c r="I18" s="376" t="n">
         <v>9</v>
       </c>
-      <c r="J18" s="371" t="inlineStr">
+      <c r="J18" s="377" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="K18" s="362" t="inlineStr">
+      <c r="K18" s="368" t="inlineStr">
         <is>
           <t>Re-engagement email</t>
         </is>
       </c>
     </row>
     <row r="19" ht="18" customHeight="1">
-      <c r="A19" s="353" t="inlineStr">
+      <c r="A19" s="358" t="inlineStr">
         <is>
           <t>C-015</t>
         </is>
       </c>
-      <c r="B19" s="371" t="inlineStr">
+      <c r="B19" s="377" t="inlineStr">
         <is>
           <t>Silver</t>
         </is>
@@ -17617,25 +17674,25 @@
       <c r="C19" s="271" t="n">
         <v>45</v>
       </c>
-      <c r="D19" s="367" t="n">
+      <c r="D19" s="373" t="n">
         <v>3</v>
       </c>
       <c r="E19" s="271" t="n">
         <v>5</v>
       </c>
-      <c r="F19" s="368" t="n">
+      <c r="F19" s="374" t="n">
         <v>3</v>
       </c>
-      <c r="G19" s="357" t="n">
+      <c r="G19" s="362" t="n">
         <v>175.94</v>
       </c>
-      <c r="H19" s="369" t="n">
+      <c r="H19" s="375" t="n">
         <v>3</v>
       </c>
-      <c r="I19" s="370" t="n">
+      <c r="I19" s="376" t="n">
         <v>9</v>
       </c>
-      <c r="J19" s="371" t="inlineStr">
+      <c r="J19" s="377" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
@@ -17647,55 +17704,55 @@
       </c>
     </row>
     <row r="20" ht="18" customHeight="1">
-      <c r="A20" s="359" t="inlineStr">
+      <c r="A20" s="365" t="inlineStr">
         <is>
           <t>C-016</t>
         </is>
       </c>
-      <c r="B20" s="371" t="inlineStr">
+      <c r="B20" s="377" t="inlineStr">
         <is>
           <t>Silver</t>
         </is>
       </c>
-      <c r="C20" s="360" t="n">
+      <c r="C20" s="366" t="n">
         <v>48</v>
       </c>
-      <c r="D20" s="367" t="n">
+      <c r="D20" s="373" t="n">
         <v>3</v>
       </c>
-      <c r="E20" s="360" t="n">
+      <c r="E20" s="366" t="n">
         <v>4</v>
       </c>
-      <c r="F20" s="368" t="n">
+      <c r="F20" s="374" t="n">
         <v>3</v>
       </c>
-      <c r="G20" s="361" t="n">
+      <c r="G20" s="367" t="n">
         <v>167.96</v>
       </c>
-      <c r="H20" s="369" t="n">
+      <c r="H20" s="375" t="n">
         <v>3</v>
       </c>
-      <c r="I20" s="370" t="n">
+      <c r="I20" s="376" t="n">
         <v>9</v>
       </c>
-      <c r="J20" s="371" t="inlineStr">
+      <c r="J20" s="377" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="K20" s="362" t="inlineStr">
+      <c r="K20" s="368" t="inlineStr">
         <is>
           <t>Newsletter highlight</t>
         </is>
       </c>
     </row>
     <row r="21" ht="18" customHeight="1">
-      <c r="A21" s="353" t="inlineStr">
+      <c r="A21" s="358" t="inlineStr">
         <is>
           <t>C-017</t>
         </is>
       </c>
-      <c r="B21" s="371" t="inlineStr">
+      <c r="B21" s="377" t="inlineStr">
         <is>
           <t>Silver</t>
         </is>
@@ -17703,25 +17760,25 @@
       <c r="C21" s="271" t="n">
         <v>52</v>
       </c>
-      <c r="D21" s="367" t="n">
+      <c r="D21" s="373" t="n">
         <v>3</v>
       </c>
       <c r="E21" s="271" t="n">
         <v>4</v>
       </c>
-      <c r="F21" s="368" t="n">
+      <c r="F21" s="374" t="n">
         <v>3</v>
       </c>
-      <c r="G21" s="357" t="n">
+      <c r="G21" s="362" t="n">
         <v>159.96</v>
       </c>
-      <c r="H21" s="369" t="n">
+      <c r="H21" s="375" t="n">
         <v>3</v>
       </c>
-      <c r="I21" s="370" t="n">
+      <c r="I21" s="376" t="n">
         <v>9</v>
       </c>
-      <c r="J21" s="371" t="inlineStr">
+      <c r="J21" s="377" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
@@ -17733,55 +17790,55 @@
       </c>
     </row>
     <row r="22" ht="18" customHeight="1">
-      <c r="A22" s="359" t="inlineStr">
+      <c r="A22" s="365" t="inlineStr">
         <is>
           <t>C-018</t>
         </is>
       </c>
-      <c r="B22" s="371" t="inlineStr">
+      <c r="B22" s="377" t="inlineStr">
         <is>
           <t>Silver</t>
         </is>
       </c>
-      <c r="C22" s="360" t="n">
+      <c r="C22" s="366" t="n">
         <v>55</v>
       </c>
-      <c r="D22" s="367" t="n">
+      <c r="D22" s="373" t="n">
         <v>3</v>
       </c>
-      <c r="E22" s="360" t="n">
+      <c r="E22" s="366" t="n">
         <v>4</v>
       </c>
-      <c r="F22" s="368" t="n">
+      <c r="F22" s="374" t="n">
         <v>3</v>
       </c>
-      <c r="G22" s="361" t="n">
+      <c r="G22" s="367" t="n">
         <v>148.2</v>
       </c>
-      <c r="H22" s="369" t="n">
+      <c r="H22" s="375" t="n">
         <v>3</v>
       </c>
-      <c r="I22" s="370" t="n">
+      <c r="I22" s="376" t="n">
         <v>9</v>
       </c>
-      <c r="J22" s="371" t="inlineStr">
+      <c r="J22" s="377" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="K22" s="362" t="inlineStr">
+      <c r="K22" s="368" t="inlineStr">
         <is>
           <t>Social proof campaign</t>
         </is>
       </c>
     </row>
     <row r="23" ht="18" customHeight="1">
-      <c r="A23" s="353" t="inlineStr">
+      <c r="A23" s="358" t="inlineStr">
         <is>
           <t>C-019</t>
         </is>
       </c>
-      <c r="B23" s="371" t="inlineStr">
+      <c r="B23" s="377" t="inlineStr">
         <is>
           <t>Silver</t>
         </is>
@@ -17789,25 +17846,25 @@
       <c r="C23" s="271" t="n">
         <v>59</v>
       </c>
-      <c r="D23" s="367" t="n">
+      <c r="D23" s="373" t="n">
         <v>3</v>
       </c>
       <c r="E23" s="271" t="n">
         <v>3</v>
       </c>
-      <c r="F23" s="372" t="n">
+      <c r="F23" s="378" t="n">
         <v>2</v>
       </c>
-      <c r="G23" s="357" t="n">
+      <c r="G23" s="362" t="n">
         <v>134.9</v>
       </c>
-      <c r="H23" s="369" t="n">
+      <c r="H23" s="375" t="n">
         <v>3</v>
       </c>
-      <c r="I23" s="370" t="n">
+      <c r="I23" s="376" t="n">
         <v>8</v>
       </c>
-      <c r="J23" s="371" t="inlineStr">
+      <c r="J23" s="377" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
@@ -17819,55 +17876,55 @@
       </c>
     </row>
     <row r="24" ht="18" customHeight="1">
-      <c r="A24" s="359" t="inlineStr">
+      <c r="A24" s="365" t="inlineStr">
         <is>
           <t>C-020</t>
         </is>
       </c>
-      <c r="B24" s="371" t="inlineStr">
+      <c r="B24" s="377" t="inlineStr">
         <is>
           <t>Silver</t>
         </is>
       </c>
-      <c r="C24" s="360" t="n">
+      <c r="C24" s="366" t="n">
         <v>63</v>
       </c>
-      <c r="D24" s="373" t="n">
+      <c r="D24" s="379" t="n">
         <v>2</v>
       </c>
-      <c r="E24" s="360" t="n">
+      <c r="E24" s="366" t="n">
         <v>3</v>
       </c>
-      <c r="F24" s="372" t="n">
+      <c r="F24" s="378" t="n">
         <v>2</v>
       </c>
-      <c r="G24" s="361" t="n">
+      <c r="G24" s="367" t="n">
         <v>124</v>
       </c>
-      <c r="H24" s="369" t="n">
+      <c r="H24" s="375" t="n">
         <v>3</v>
       </c>
-      <c r="I24" s="370" t="n">
+      <c r="I24" s="376" t="n">
         <v>7</v>
       </c>
-      <c r="J24" s="371" t="inlineStr">
+      <c r="J24" s="377" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="K24" s="362" t="inlineStr">
+      <c r="K24" s="368" t="inlineStr">
         <is>
           <t>Browse reminder</t>
         </is>
       </c>
     </row>
     <row r="25" ht="18" customHeight="1">
-      <c r="A25" s="353" t="inlineStr">
+      <c r="A25" s="358" t="inlineStr">
         <is>
           <t>C-025</t>
         </is>
       </c>
-      <c r="B25" s="374" t="inlineStr">
+      <c r="B25" s="380" t="inlineStr">
         <is>
           <t>Silver</t>
         </is>
@@ -17875,25 +17932,25 @@
       <c r="C25" s="271" t="n">
         <v>92</v>
       </c>
-      <c r="D25" s="373" t="n">
+      <c r="D25" s="379" t="n">
         <v>2</v>
       </c>
       <c r="E25" s="271" t="n">
         <v>2</v>
       </c>
-      <c r="F25" s="372" t="n">
+      <c r="F25" s="378" t="n">
         <v>2</v>
       </c>
-      <c r="G25" s="357" t="n">
+      <c r="G25" s="362" t="n">
         <v>91.98</v>
       </c>
-      <c r="H25" s="375" t="n">
+      <c r="H25" s="381" t="n">
         <v>2</v>
       </c>
-      <c r="I25" s="376" t="n">
+      <c r="I25" s="382" t="n">
         <v>6</v>
       </c>
-      <c r="J25" s="374" t="inlineStr">
+      <c r="J25" s="380" t="inlineStr">
         <is>
           <t>At Risk</t>
         </is>
@@ -17905,55 +17962,55 @@
       </c>
     </row>
     <row r="26" ht="18" customHeight="1">
-      <c r="A26" s="359" t="inlineStr">
+      <c r="A26" s="365" t="inlineStr">
         <is>
           <t>C-026</t>
         </is>
       </c>
-      <c r="B26" s="374" t="inlineStr">
+      <c r="B26" s="380" t="inlineStr">
         <is>
           <t>Silver</t>
         </is>
       </c>
-      <c r="C26" s="360" t="n">
+      <c r="C26" s="366" t="n">
         <v>101</v>
       </c>
-      <c r="D26" s="373" t="n">
+      <c r="D26" s="379" t="n">
         <v>2</v>
       </c>
-      <c r="E26" s="360" t="n">
+      <c r="E26" s="366" t="n">
         <v>2</v>
       </c>
-      <c r="F26" s="372" t="n">
+      <c r="F26" s="378" t="n">
         <v>2</v>
       </c>
-      <c r="G26" s="361" t="n">
+      <c r="G26" s="367" t="n">
         <v>84.98</v>
       </c>
-      <c r="H26" s="375" t="n">
+      <c r="H26" s="381" t="n">
         <v>2</v>
       </c>
-      <c r="I26" s="376" t="n">
+      <c r="I26" s="382" t="n">
         <v>6</v>
       </c>
-      <c r="J26" s="374" t="inlineStr">
+      <c r="J26" s="380" t="inlineStr">
         <is>
           <t>At Risk</t>
         </is>
       </c>
-      <c r="K26" s="362" t="inlineStr">
+      <c r="K26" s="368" t="inlineStr">
         <is>
           <t>Personalised outreach</t>
         </is>
       </c>
     </row>
     <row r="27" ht="18" customHeight="1">
-      <c r="A27" s="353" t="inlineStr">
+      <c r="A27" s="358" t="inlineStr">
         <is>
           <t>C-027</t>
         </is>
       </c>
-      <c r="B27" s="374" t="inlineStr">
+      <c r="B27" s="380" t="inlineStr">
         <is>
           <t>Bronze</t>
         </is>
@@ -17961,25 +18018,25 @@
       <c r="C27" s="271" t="n">
         <v>112</v>
       </c>
-      <c r="D27" s="373" t="n">
+      <c r="D27" s="379" t="n">
         <v>2</v>
       </c>
       <c r="E27" s="271" t="n">
         <v>2</v>
       </c>
-      <c r="F27" s="372" t="n">
+      <c r="F27" s="378" t="n">
         <v>2</v>
       </c>
-      <c r="G27" s="357" t="n">
+      <c r="G27" s="362" t="n">
         <v>76.98</v>
       </c>
-      <c r="H27" s="375" t="n">
+      <c r="H27" s="381" t="n">
         <v>2</v>
       </c>
-      <c r="I27" s="376" t="n">
+      <c r="I27" s="382" t="n">
         <v>6</v>
       </c>
-      <c r="J27" s="374" t="inlineStr">
+      <c r="J27" s="380" t="inlineStr">
         <is>
           <t>At Risk</t>
         </is>
@@ -17991,55 +18048,55 @@
       </c>
     </row>
     <row r="28" ht="18" customHeight="1">
-      <c r="A28" s="359" t="inlineStr">
+      <c r="A28" s="365" t="inlineStr">
         <is>
           <t>C-028</t>
         </is>
       </c>
-      <c r="B28" s="374" t="inlineStr">
+      <c r="B28" s="380" t="inlineStr">
         <is>
           <t>Bronze</t>
         </is>
       </c>
-      <c r="C28" s="360" t="n">
+      <c r="C28" s="366" t="n">
         <v>121</v>
       </c>
-      <c r="D28" s="373" t="n">
+      <c r="D28" s="379" t="n">
         <v>1</v>
       </c>
-      <c r="E28" s="360" t="n">
+      <c r="E28" s="366" t="n">
         <v>2</v>
       </c>
-      <c r="F28" s="372" t="n">
+      <c r="F28" s="378" t="n">
         <v>2</v>
       </c>
-      <c r="G28" s="361" t="n">
+      <c r="G28" s="367" t="n">
         <v>69.98</v>
       </c>
-      <c r="H28" s="375" t="n">
+      <c r="H28" s="381" t="n">
         <v>2</v>
       </c>
-      <c r="I28" s="376" t="n">
+      <c r="I28" s="382" t="n">
         <v>5</v>
       </c>
-      <c r="J28" s="374" t="inlineStr">
+      <c r="J28" s="380" t="inlineStr">
         <is>
           <t>At Risk</t>
         </is>
       </c>
-      <c r="K28" s="362" t="inlineStr">
+      <c r="K28" s="368" t="inlineStr">
         <is>
           <t>Limited-time offer</t>
         </is>
       </c>
     </row>
     <row r="29" ht="18" customHeight="1">
-      <c r="A29" s="353" t="inlineStr">
+      <c r="A29" s="358" t="inlineStr">
         <is>
           <t>C-029</t>
         </is>
       </c>
-      <c r="B29" s="374" t="inlineStr">
+      <c r="B29" s="380" t="inlineStr">
         <is>
           <t>Bronze</t>
         </is>
@@ -18047,25 +18104,25 @@
       <c r="C29" s="271" t="n">
         <v>134</v>
       </c>
-      <c r="D29" s="373" t="n">
+      <c r="D29" s="379" t="n">
         <v>1</v>
       </c>
       <c r="E29" s="271" t="n">
         <v>1</v>
       </c>
-      <c r="F29" s="372" t="n">
+      <c r="F29" s="378" t="n">
         <v>1</v>
       </c>
-      <c r="G29" s="357" t="n">
+      <c r="G29" s="362" t="n">
         <v>62.99</v>
       </c>
-      <c r="H29" s="375" t="n">
+      <c r="H29" s="381" t="n">
         <v>2</v>
       </c>
-      <c r="I29" s="376" t="n">
+      <c r="I29" s="382" t="n">
         <v>4</v>
       </c>
-      <c r="J29" s="374" t="inlineStr">
+      <c r="J29" s="380" t="inlineStr">
         <is>
           <t>At Risk</t>
         </is>
@@ -18077,55 +18134,55 @@
       </c>
     </row>
     <row r="30" ht="18" customHeight="1">
-      <c r="A30" s="359" t="inlineStr">
+      <c r="A30" s="365" t="inlineStr">
         <is>
           <t>C-030</t>
         </is>
       </c>
-      <c r="B30" s="374" t="inlineStr">
+      <c r="B30" s="380" t="inlineStr">
         <is>
           <t>Bronze</t>
         </is>
       </c>
-      <c r="C30" s="360" t="n">
+      <c r="C30" s="366" t="n">
         <v>143</v>
       </c>
-      <c r="D30" s="373" t="n">
+      <c r="D30" s="379" t="n">
         <v>1</v>
       </c>
-      <c r="E30" s="360" t="n">
+      <c r="E30" s="366" t="n">
         <v>1</v>
       </c>
-      <c r="F30" s="372" t="n">
+      <c r="F30" s="378" t="n">
         <v>1</v>
       </c>
-      <c r="G30" s="361" t="n">
+      <c r="G30" s="367" t="n">
         <v>57.99</v>
       </c>
-      <c r="H30" s="375" t="n">
+      <c r="H30" s="381" t="n">
         <v>2</v>
       </c>
-      <c r="I30" s="376" t="n">
+      <c r="I30" s="382" t="n">
         <v>4</v>
       </c>
-      <c r="J30" s="374" t="inlineStr">
+      <c r="J30" s="380" t="inlineStr">
         <is>
           <t>At Risk</t>
         </is>
       </c>
-      <c r="K30" s="362" t="inlineStr">
+      <c r="K30" s="368" t="inlineStr">
         <is>
           <t>Social retargeting</t>
         </is>
       </c>
     </row>
     <row r="31" ht="18" customHeight="1">
-      <c r="A31" s="353" t="inlineStr">
+      <c r="A31" s="358" t="inlineStr">
         <is>
           <t>C-035</t>
         </is>
       </c>
-      <c r="B31" s="377" t="inlineStr">
+      <c r="B31" s="383" t="inlineStr">
         <is>
           <t>Bronze</t>
         </is>
@@ -18133,25 +18190,25 @@
       <c r="C31" s="271" t="n">
         <v>201</v>
       </c>
-      <c r="D31" s="373" t="n">
+      <c r="D31" s="379" t="n">
         <v>1</v>
       </c>
       <c r="E31" s="271" t="n">
         <v>1</v>
       </c>
-      <c r="F31" s="372" t="n">
+      <c r="F31" s="378" t="n">
         <v>1</v>
       </c>
-      <c r="G31" s="357" t="n">
+      <c r="G31" s="362" t="n">
         <v>34.99</v>
       </c>
-      <c r="H31" s="375" t="n">
+      <c r="H31" s="381" t="n">
         <v>1</v>
       </c>
-      <c r="I31" s="376" t="n">
+      <c r="I31" s="382" t="n">
         <v>3</v>
       </c>
-      <c r="J31" s="377" t="inlineStr">
+      <c r="J31" s="383" t="inlineStr">
         <is>
           <t>Lost</t>
         </is>
@@ -18163,55 +18220,55 @@
       </c>
     </row>
     <row r="32" ht="18" customHeight="1">
-      <c r="A32" s="359" t="inlineStr">
+      <c r="A32" s="365" t="inlineStr">
         <is>
           <t>C-036</t>
         </is>
       </c>
-      <c r="B32" s="377" t="inlineStr">
+      <c r="B32" s="383" t="inlineStr">
         <is>
           <t>Bronze</t>
         </is>
       </c>
-      <c r="C32" s="360" t="n">
+      <c r="C32" s="366" t="n">
         <v>214</v>
       </c>
-      <c r="D32" s="373" t="n">
+      <c r="D32" s="379" t="n">
         <v>1</v>
       </c>
-      <c r="E32" s="360" t="n">
+      <c r="E32" s="366" t="n">
         <v>1</v>
       </c>
-      <c r="F32" s="372" t="n">
+      <c r="F32" s="378" t="n">
         <v>1</v>
       </c>
-      <c r="G32" s="361" t="n">
+      <c r="G32" s="367" t="n">
         <v>32.99</v>
       </c>
-      <c r="H32" s="375" t="n">
+      <c r="H32" s="381" t="n">
         <v>1</v>
       </c>
-      <c r="I32" s="376" t="n">
+      <c r="I32" s="382" t="n">
         <v>3</v>
       </c>
-      <c r="J32" s="377" t="inlineStr">
+      <c r="J32" s="383" t="inlineStr">
         <is>
           <t>Lost</t>
         </is>
       </c>
-      <c r="K32" s="362" t="inlineStr">
+      <c r="K32" s="368" t="inlineStr">
         <is>
           <t>Final reactivation</t>
         </is>
       </c>
     </row>
     <row r="33" ht="18" customHeight="1">
-      <c r="A33" s="353" t="inlineStr">
+      <c r="A33" s="358" t="inlineStr">
         <is>
           <t>C-037</t>
         </is>
       </c>
-      <c r="B33" s="377" t="inlineStr">
+      <c r="B33" s="383" t="inlineStr">
         <is>
           <t>Bronze</t>
         </is>
@@ -18219,25 +18276,25 @@
       <c r="C33" s="271" t="n">
         <v>223</v>
       </c>
-      <c r="D33" s="373" t="n">
+      <c r="D33" s="379" t="n">
         <v>1</v>
       </c>
       <c r="E33" s="271" t="n">
         <v>1</v>
       </c>
-      <c r="F33" s="372" t="n">
+      <c r="F33" s="378" t="n">
         <v>1</v>
       </c>
-      <c r="G33" s="357" t="n">
+      <c r="G33" s="362" t="n">
         <v>29.99</v>
       </c>
-      <c r="H33" s="375" t="n">
+      <c r="H33" s="381" t="n">
         <v>1</v>
       </c>
-      <c r="I33" s="376" t="n">
+      <c r="I33" s="382" t="n">
         <v>3</v>
       </c>
-      <c r="J33" s="377" t="inlineStr">
+      <c r="J33" s="383" t="inlineStr">
         <is>
           <t>Lost</t>
         </is>
@@ -18249,150 +18306,150 @@
       </c>
     </row>
     <row r="34" ht="18" customHeight="1">
-      <c r="A34" s="359" t="inlineStr">
+      <c r="A34" s="365" t="inlineStr">
         <is>
           <t>C-038</t>
         </is>
       </c>
-      <c r="B34" s="377" t="inlineStr">
+      <c r="B34" s="383" t="inlineStr">
         <is>
           <t>Bronze</t>
         </is>
       </c>
-      <c r="C34" s="360" t="n">
+      <c r="C34" s="366" t="n">
         <v>238</v>
       </c>
-      <c r="D34" s="373" t="n">
+      <c r="D34" s="379" t="n">
         <v>1</v>
       </c>
-      <c r="E34" s="360" t="n">
+      <c r="E34" s="366" t="n">
         <v>1</v>
       </c>
-      <c r="F34" s="372" t="n">
+      <c r="F34" s="378" t="n">
         <v>1</v>
       </c>
-      <c r="G34" s="361" t="n">
+      <c r="G34" s="367" t="n">
         <v>27.99</v>
       </c>
-      <c r="H34" s="375" t="n">
+      <c r="H34" s="381" t="n">
         <v>1</v>
       </c>
-      <c r="I34" s="376" t="n">
+      <c r="I34" s="382" t="n">
         <v>3</v>
       </c>
-      <c r="J34" s="377" t="inlineStr">
+      <c r="J34" s="383" t="inlineStr">
         <is>
           <t>Lost</t>
         </is>
       </c>
-      <c r="K34" s="362" t="inlineStr">
+      <c r="K34" s="368" t="inlineStr">
         <is>
           <t>Archive segment</t>
         </is>
       </c>
     </row>
     <row r="37" ht="20" customHeight="1">
-      <c r="A37" s="378" t="inlineStr">
+      <c r="A37" s="384" t="inlineStr">
         <is>
           <t>SEGMENT SUMMARY</t>
         </is>
       </c>
     </row>
     <row r="38" ht="18" customHeight="1">
-      <c r="A38" s="354" t="inlineStr">
+      <c r="A38" s="359" t="inlineStr">
         <is>
           <t>Champion</t>
         </is>
       </c>
-      <c r="B38" s="379" t="n">
+      <c r="B38" s="385" t="n">
         <v>5</v>
       </c>
-      <c r="C38" s="380" t="inlineStr">
+      <c r="C38" s="386" t="inlineStr">
         <is>
           <t>892–149 avg spend</t>
         </is>
       </c>
-      <c r="E38" s="381" t="inlineStr">
+      <c r="E38" s="387" t="inlineStr">
         <is>
           <t>Top 5 Platinum customers · Revenue: $3,418 · Avg RFM: 14.2</t>
         </is>
       </c>
     </row>
     <row r="39" ht="18" customHeight="1">
-      <c r="A39" s="365" t="inlineStr">
+      <c r="A39" s="371" t="inlineStr">
         <is>
           <t>Loyal</t>
         </is>
       </c>
-      <c r="B39" s="379" t="n">
+      <c r="B39" s="385" t="n">
         <v>8</v>
       </c>
-      <c r="C39" s="380" t="inlineStr">
+      <c r="C39" s="386" t="inlineStr">
         <is>
           <t>419–218 avg spend</t>
         </is>
       </c>
-      <c r="E39" s="381" t="inlineStr">
+      <c r="E39" s="387" t="inlineStr">
         <is>
           <t>Gold tier regulars · Revenue: $2,361 · Avg RFM: 10.8</t>
         </is>
       </c>
     </row>
     <row r="40" ht="18" customHeight="1">
-      <c r="A40" s="371" t="inlineStr">
+      <c r="A40" s="377" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="B40" s="379" t="n">
+      <c r="B40" s="385" t="n">
         <v>7</v>
       </c>
-      <c r="C40" s="380" t="inlineStr">
+      <c r="C40" s="386" t="inlineStr">
         <is>
           <t>189–124 avg spend</t>
         </is>
       </c>
-      <c r="E40" s="381" t="inlineStr">
+      <c r="E40" s="387" t="inlineStr">
         <is>
           <t>Silver casuals · Revenue: $1,101 · Avg RFM: 8.1</t>
         </is>
       </c>
     </row>
     <row r="41" ht="18" customHeight="1">
-      <c r="A41" s="374" t="inlineStr">
+      <c r="A41" s="380" t="inlineStr">
         <is>
           <t>At Risk</t>
         </is>
       </c>
-      <c r="B41" s="379" t="n">
+      <c r="B41" s="385" t="n">
         <v>6</v>
       </c>
-      <c r="C41" s="380" t="inlineStr">
+      <c r="C41" s="386" t="inlineStr">
         <is>
           <t>92–58 avg spend</t>
         </is>
       </c>
-      <c r="E41" s="381" t="inlineStr">
+      <c r="E41" s="387" t="inlineStr">
         <is>
           <t>Declining frequency · Revenue:  $444 · Avg RFM: 5.3</t>
         </is>
       </c>
     </row>
     <row r="42" ht="18" customHeight="1">
-      <c r="A42" s="377" t="inlineStr">
+      <c r="A42" s="383" t="inlineStr">
         <is>
           <t>Lost</t>
         </is>
       </c>
-      <c r="B42" s="379" t="n">
+      <c r="B42" s="385" t="n">
         <v>4</v>
       </c>
-      <c r="C42" s="380" t="inlineStr">
+      <c r="C42" s="386" t="inlineStr">
         <is>
           <t>35–28 avg spend</t>
         </is>
       </c>
-      <c r="E42" s="381" t="inlineStr">
+      <c r="E42" s="387" t="inlineStr">
         <is>
           <t>No recent activity  · Revenue:  $126 · Avg RFM: 3.0</t>
         </is>

</xml_diff>